<commit_message>
Update Identifier slicing a6f738ba786046b09317a60423b31666b4379010
</commit_message>
<xml_diff>
--- a/449-contenu-fhir---ajout-des-objets-presenceabsence-et-repas/ig/StructureDefinition-tddui-observation-repas.xlsx
+++ b/449-contenu-fhir---ajout-des-objets-presenceabsence-et-repas/ig/StructureDefinition-tddui-observation-repas.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2436" uniqueCount="522">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2475" uniqueCount="533">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-03T14:26:22+00:00</t>
+    <t>2026-06-09T13:44:39+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -535,6 +535,10 @@
     <t>Allows observations to be distinguished and referenced.</t>
   </si>
   <si>
+    <t xml:space="preserve">pattern:type}
+</t>
+  </si>
+  <si>
     <t>idRepas</t>
   </si>
   <si>
@@ -548,6 +552,12 @@
   </si>
   <si>
     <t>FiveWs.identifier</t>
+  </si>
+  <si>
+    <t>Observation.identifier:idRepas</t>
+  </si>
+  <si>
+    <t>Observation.identifier:idRepas.id</t>
   </si>
   <si>
     <t>Observation.identifier.id</t>
@@ -569,6 +579,9 @@
     <t>n/a</t>
   </si>
   <si>
+    <t>Observation.identifier:idRepas.extension</t>
+  </si>
+  <si>
     <t>Observation.identifier.extension</t>
   </si>
   <si>
@@ -584,6 +597,9 @@
     <t>Element.extension</t>
   </si>
   <si>
+    <t>Observation.identifier:idRepas.use</t>
+  </si>
+  <si>
     <t>Observation.identifier.use</t>
   </si>
   <si>
@@ -612,6 +628,9 @@
   </si>
   <si>
     <t>Role.code or implied by context</t>
+  </si>
+  <si>
+    <t>Observation.identifier:idRepas.type</t>
   </si>
   <si>
     <t>Observation.identifier.type</t>
@@ -633,6 +652,14 @@
     <t>Allows users to make use of identifiers when the identifier system is not known.</t>
   </si>
   <si>
+    <t>&lt;valueCodeableConcept xmlns="http://hl7.org/fhir"&gt;
+  &lt;coding&gt;
+    &lt;system value="https://interop.esante.gouv.fr/ig/fhir/tddui/CodeSystem/tddui-observation-identifier"/&gt;
+    &lt;code value="REP"/&gt;
+  &lt;/coding&gt;
+&lt;/valueCodeableConcept&gt;</t>
+  </si>
+  <si>
     <t>extensible</t>
   </si>
   <si>
@@ -648,6 +675,9 @@
     <t>CX.5</t>
   </si>
   <si>
+    <t>Observation.identifier:idRepas.system</t>
+  </si>
+  <si>
     <t>Observation.identifier.system</t>
   </si>
   <si>
@@ -678,6 +708,9 @@
     <t>II.root or Role.id.root</t>
   </si>
   <si>
+    <t>Observation.identifier:idRepas.value</t>
+  </si>
+  <si>
     <t>Observation.identifier.value</t>
   </si>
   <si>
@@ -700,6 +733,9 @@
   </si>
   <si>
     <t>II.extension or II.root if system indicates OID or GUID (Or Role.id.extension or root)</t>
+  </si>
+  <si>
+    <t>Observation.identifier:idRepas.period</t>
   </si>
   <si>
     <t>Observation.identifier.period</t>
@@ -722,6 +758,9 @@
   </si>
   <si>
     <t>Role.effectiveTime or implied by context</t>
+  </si>
+  <si>
+    <t>Observation.identifier:idRepas.assigner</t>
   </si>
   <si>
     <t>Observation.identifier.assigner</t>
@@ -1952,7 +1991,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AQ61"/>
+  <dimension ref="A1:AQ62"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
     <col min="1" max="1" width="38.30078125" customWidth="true" bestFit="true"/>
@@ -3372,7 +3411,7 @@
         <v>95</v>
       </c>
       <c r="G12" t="s" s="2">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="H12" t="s" s="2">
         <v>83</v>
@@ -3431,16 +3470,14 @@
         <v>83</v>
       </c>
       <c r="AB12" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AC12" t="s" s="2">
-        <v>83</v>
-      </c>
+        <v>166</v>
+      </c>
+      <c r="AC12" s="2"/>
       <c r="AD12" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AE12" t="s" s="2">
-        <v>83</v>
+        <v>144</v>
       </c>
       <c r="AF12" t="s" s="2">
         <v>161</v>
@@ -3458,22 +3495,22 @@
         <v>107</v>
       </c>
       <c r="AK12" t="s" s="2">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="AL12" t="s" s="2">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="AM12" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AN12" t="s" s="2">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="AO12" t="s" s="2">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="AP12" t="s" s="2">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="AQ12" t="s" s="2">
         <v>83</v>
@@ -3481,18 +3518,20 @@
     </row>
     <row r="13">
       <c r="A13" t="s" s="2">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>171</v>
-      </c>
-      <c r="C13" s="2"/>
+        <v>161</v>
+      </c>
+      <c r="C13" t="s" s="2">
+        <v>167</v>
+      </c>
       <c r="D13" t="s" s="2">
         <v>83</v>
       </c>
       <c r="E13" s="2"/>
       <c r="F13" t="s" s="2">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="G13" t="s" s="2">
         <v>95</v>
@@ -3504,19 +3543,21 @@
         <v>83</v>
       </c>
       <c r="J13" t="s" s="2">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="K13" t="s" s="2">
-        <v>172</v>
+        <v>162</v>
       </c>
       <c r="L13" t="s" s="2">
-        <v>173</v>
+        <v>163</v>
       </c>
       <c r="M13" t="s" s="2">
-        <v>174</v>
+        <v>164</v>
       </c>
       <c r="N13" s="2"/>
-      <c r="O13" s="2"/>
+      <c r="O13" t="s" s="2">
+        <v>165</v>
+      </c>
       <c r="P13" t="s" s="2">
         <v>83</v>
       </c>
@@ -3564,37 +3605,37 @@
         <v>83</v>
       </c>
       <c r="AF13" t="s" s="2">
-        <v>175</v>
+        <v>161</v>
       </c>
       <c r="AG13" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH13" t="s" s="2">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="AI13" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AJ13" t="s" s="2">
-        <v>83</v>
+        <v>107</v>
       </c>
       <c r="AK13" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AL13" t="s" s="2">
-        <v>83</v>
+        <v>168</v>
       </c>
       <c r="AM13" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AN13" t="s" s="2">
-        <v>83</v>
+        <v>169</v>
       </c>
       <c r="AO13" t="s" s="2">
-        <v>176</v>
+        <v>170</v>
       </c>
       <c r="AP13" t="s" s="2">
-        <v>83</v>
+        <v>171</v>
       </c>
       <c r="AQ13" t="s" s="2">
         <v>83</v>
@@ -3602,21 +3643,21 @@
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" t="s" s="2">
-        <v>155</v>
+        <v>83</v>
       </c>
       <c r="E14" s="2"/>
       <c r="F14" t="s" s="2">
         <v>81</v>
       </c>
       <c r="G14" t="s" s="2">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="H14" t="s" s="2">
         <v>83</v>
@@ -3628,17 +3669,15 @@
         <v>83</v>
       </c>
       <c r="K14" t="s" s="2">
-        <v>140</v>
+        <v>175</v>
       </c>
       <c r="L14" t="s" s="2">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="M14" t="s" s="2">
-        <v>179</v>
-      </c>
-      <c r="N14" t="s" s="2">
-        <v>158</v>
-      </c>
+        <v>177</v>
+      </c>
+      <c r="N14" s="2"/>
       <c r="O14" s="2"/>
       <c r="P14" t="s" s="2">
         <v>83</v>
@@ -3675,31 +3714,31 @@
         <v>83</v>
       </c>
       <c r="AB14" t="s" s="2">
-        <v>143</v>
+        <v>83</v>
       </c>
       <c r="AC14" t="s" s="2">
-        <v>180</v>
+        <v>83</v>
       </c>
       <c r="AD14" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AE14" t="s" s="2">
-        <v>144</v>
+        <v>83</v>
       </c>
       <c r="AF14" t="s" s="2">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="AG14" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH14" t="s" s="2">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="AI14" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AJ14" t="s" s="2">
-        <v>146</v>
+        <v>83</v>
       </c>
       <c r="AK14" t="s" s="2">
         <v>83</v>
@@ -3714,7 +3753,7 @@
         <v>83</v>
       </c>
       <c r="AO14" t="s" s="2">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="AP14" t="s" s="2">
         <v>83</v>
@@ -3725,46 +3764,44 @@
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" t="s" s="2">
-        <v>83</v>
+        <v>155</v>
       </c>
       <c r="E15" s="2"/>
       <c r="F15" t="s" s="2">
         <v>81</v>
       </c>
       <c r="G15" t="s" s="2">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="H15" t="s" s="2">
         <v>83</v>
       </c>
       <c r="I15" t="s" s="2">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="J15" t="s" s="2">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="K15" t="s" s="2">
-        <v>115</v>
+        <v>140</v>
       </c>
       <c r="L15" t="s" s="2">
+        <v>182</v>
+      </c>
+      <c r="M15" t="s" s="2">
         <v>183</v>
       </c>
-      <c r="M15" t="s" s="2">
-        <v>184</v>
-      </c>
       <c r="N15" t="s" s="2">
-        <v>185</v>
-      </c>
-      <c r="O15" t="s" s="2">
-        <v>186</v>
-      </c>
+        <v>158</v>
+      </c>
+      <c r="O15" s="2"/>
       <c r="P15" t="s" s="2">
         <v>83</v>
       </c>
@@ -3788,43 +3825,43 @@
         <v>83</v>
       </c>
       <c r="X15" t="s" s="2">
-        <v>187</v>
+        <v>83</v>
       </c>
       <c r="Y15" t="s" s="2">
-        <v>188</v>
+        <v>83</v>
       </c>
       <c r="Z15" t="s" s="2">
-        <v>189</v>
+        <v>83</v>
       </c>
       <c r="AA15" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AB15" t="s" s="2">
-        <v>83</v>
+        <v>143</v>
       </c>
       <c r="AC15" t="s" s="2">
-        <v>83</v>
+        <v>184</v>
       </c>
       <c r="AD15" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AE15" t="s" s="2">
-        <v>83</v>
+        <v>144</v>
       </c>
       <c r="AF15" t="s" s="2">
-        <v>190</v>
+        <v>185</v>
       </c>
       <c r="AG15" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH15" t="s" s="2">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="AI15" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AJ15" t="s" s="2">
-        <v>107</v>
+        <v>146</v>
       </c>
       <c r="AK15" t="s" s="2">
         <v>83</v>
@@ -3836,10 +3873,10 @@
         <v>83</v>
       </c>
       <c r="AN15" t="s" s="2">
-        <v>138</v>
+        <v>83</v>
       </c>
       <c r="AO15" t="s" s="2">
-        <v>191</v>
+        <v>179</v>
       </c>
       <c r="AP15" t="s" s="2">
         <v>83</v>
@@ -3850,10 +3887,10 @@
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>192</v>
+        <v>187</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
@@ -3870,25 +3907,25 @@
         <v>83</v>
       </c>
       <c r="I16" t="s" s="2">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="J16" t="s" s="2">
         <v>96</v>
       </c>
       <c r="K16" t="s" s="2">
-        <v>193</v>
+        <v>115</v>
       </c>
       <c r="L16" t="s" s="2">
-        <v>194</v>
+        <v>188</v>
       </c>
       <c r="M16" t="s" s="2">
-        <v>195</v>
+        <v>189</v>
       </c>
       <c r="N16" t="s" s="2">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="O16" t="s" s="2">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="P16" t="s" s="2">
         <v>83</v>
@@ -3913,13 +3950,13 @@
         <v>83</v>
       </c>
       <c r="X16" t="s" s="2">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="Y16" t="s" s="2">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="Z16" t="s" s="2">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="AA16" t="s" s="2">
         <v>83</v>
@@ -3937,7 +3974,7 @@
         <v>83</v>
       </c>
       <c r="AF16" t="s" s="2">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="AG16" t="s" s="2">
         <v>81</v>
@@ -3961,10 +3998,10 @@
         <v>83</v>
       </c>
       <c r="AN16" t="s" s="2">
-        <v>202</v>
+        <v>138</v>
       </c>
       <c r="AO16" t="s" s="2">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="AP16" t="s" s="2">
         <v>83</v>
@@ -3975,10 +4012,10 @@
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -4001,19 +4038,19 @@
         <v>96</v>
       </c>
       <c r="K17" t="s" s="2">
-        <v>109</v>
+        <v>199</v>
       </c>
       <c r="L17" t="s" s="2">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="M17" t="s" s="2">
-        <v>205</v>
+        <v>201</v>
       </c>
       <c r="N17" t="s" s="2">
-        <v>206</v>
+        <v>202</v>
       </c>
       <c r="O17" t="s" s="2">
-        <v>207</v>
+        <v>203</v>
       </c>
       <c r="P17" t="s" s="2">
         <v>83</v>
@@ -4023,46 +4060,46 @@
         <v>83</v>
       </c>
       <c r="S17" t="s" s="2">
+        <v>204</v>
+      </c>
+      <c r="T17" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="U17" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="V17" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="W17" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="X17" t="s" s="2">
+        <v>205</v>
+      </c>
+      <c r="Y17" t="s" s="2">
+        <v>206</v>
+      </c>
+      <c r="Z17" t="s" s="2">
+        <v>207</v>
+      </c>
+      <c r="AA17" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AB17" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AC17" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AD17" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AE17" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AF17" t="s" s="2">
         <v>208</v>
-      </c>
-      <c r="T17" t="s" s="2">
-        <v>209</v>
-      </c>
-      <c r="U17" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="V17" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="W17" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="X17" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="Y17" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="Z17" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AA17" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AB17" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AC17" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AD17" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AE17" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AF17" t="s" s="2">
-        <v>210</v>
       </c>
       <c r="AG17" t="s" s="2">
         <v>81</v>
@@ -4086,10 +4123,10 @@
         <v>83</v>
       </c>
       <c r="AN17" t="s" s="2">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="AO17" t="s" s="2">
-        <v>212</v>
+        <v>196</v>
       </c>
       <c r="AP17" t="s" s="2">
         <v>83</v>
@@ -4100,10 +4137,10 @@
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
@@ -4126,18 +4163,20 @@
         <v>96</v>
       </c>
       <c r="K18" t="s" s="2">
-        <v>172</v>
+        <v>109</v>
       </c>
       <c r="L18" t="s" s="2">
+        <v>212</v>
+      </c>
+      <c r="M18" t="s" s="2">
+        <v>213</v>
+      </c>
+      <c r="N18" t="s" s="2">
         <v>214</v>
       </c>
-      <c r="M18" t="s" s="2">
+      <c r="O18" t="s" s="2">
         <v>215</v>
       </c>
-      <c r="N18" t="s" s="2">
-        <v>216</v>
-      </c>
-      <c r="O18" s="2"/>
       <c r="P18" t="s" s="2">
         <v>83</v>
       </c>
@@ -4146,7 +4185,7 @@
         <v>83</v>
       </c>
       <c r="S18" t="s" s="2">
-        <v>83</v>
+        <v>216</v>
       </c>
       <c r="T18" t="s" s="2">
         <v>217</v>
@@ -4226,7 +4265,7 @@
         <v>221</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
@@ -4249,7 +4288,7 @@
         <v>96</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>222</v>
+        <v>175</v>
       </c>
       <c r="L19" t="s" s="2">
         <v>223</v>
@@ -4257,7 +4296,9 @@
       <c r="M19" t="s" s="2">
         <v>224</v>
       </c>
-      <c r="N19" s="2"/>
+      <c r="N19" t="s" s="2">
+        <v>225</v>
+      </c>
       <c r="O19" s="2"/>
       <c r="P19" t="s" s="2">
         <v>83</v>
@@ -4270,7 +4311,7 @@
         <v>83</v>
       </c>
       <c r="T19" t="s" s="2">
-        <v>83</v>
+        <v>226</v>
       </c>
       <c r="U19" t="s" s="2">
         <v>83</v>
@@ -4306,7 +4347,7 @@
         <v>83</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>81</v>
@@ -4330,10 +4371,10 @@
         <v>83</v>
       </c>
       <c r="AN19" t="s" s="2">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="AO19" t="s" s="2">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="AP19" t="s" s="2">
         <v>83</v>
@@ -4344,10 +4385,10 @@
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
@@ -4370,17 +4411,15 @@
         <v>96</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>231</v>
-      </c>
-      <c r="N20" t="s" s="2">
-        <v>232</v>
-      </c>
+        <v>234</v>
+      </c>
+      <c r="N20" s="2"/>
       <c r="O20" s="2"/>
       <c r="P20" t="s" s="2">
         <v>83</v>
@@ -4429,7 +4468,7 @@
         <v>83</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>81</v>
@@ -4453,10 +4492,10 @@
         <v>83</v>
       </c>
       <c r="AN20" t="s" s="2">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="AO20" t="s" s="2">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="AP20" t="s" s="2">
         <v>83</v>
@@ -4467,21 +4506,21 @@
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>236</v>
+        <v>239</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
-        <v>237</v>
+        <v>83</v>
       </c>
       <c r="E21" s="2"/>
       <c r="F21" t="s" s="2">
         <v>81</v>
       </c>
       <c r="G21" t="s" s="2">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="H21" t="s" s="2">
         <v>83</v>
@@ -4493,18 +4532,18 @@
         <v>96</v>
       </c>
       <c r="K21" t="s" s="2">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>240</v>
-      </c>
-      <c r="N21" s="2"/>
-      <c r="O21" t="s" s="2">
-        <v>241</v>
-      </c>
+        <v>242</v>
+      </c>
+      <c r="N21" t="s" s="2">
+        <v>243</v>
+      </c>
+      <c r="O21" s="2"/>
       <c r="P21" t="s" s="2">
         <v>83</v>
       </c>
@@ -4552,13 +4591,13 @@
         <v>83</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH21" t="s" s="2">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="AI21" t="s" s="2">
         <v>83</v>
@@ -4570,16 +4609,16 @@
         <v>83</v>
       </c>
       <c r="AL21" t="s" s="2">
-        <v>242</v>
+        <v>83</v>
       </c>
       <c r="AM21" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AN21" t="s" s="2">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="AO21" t="s" s="2">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="AP21" t="s" s="2">
         <v>83</v>
@@ -4590,14 +4629,14 @@
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="E22" s="2"/>
       <c r="F22" t="s" s="2">
@@ -4616,18 +4655,18 @@
         <v>96</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>249</v>
-      </c>
-      <c r="N22" t="s" s="2">
-        <v>250</v>
-      </c>
-      <c r="O22" s="2"/>
+        <v>251</v>
+      </c>
+      <c r="N22" s="2"/>
+      <c r="O22" t="s" s="2">
+        <v>252</v>
+      </c>
       <c r="P22" t="s" s="2">
         <v>83</v>
       </c>
@@ -4675,7 +4714,7 @@
         <v>83</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>81</v>
@@ -4693,16 +4732,16 @@
         <v>83</v>
       </c>
       <c r="AL22" t="s" s="2">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="AM22" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AN22" t="s" s="2">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="AO22" t="s" s="2">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AP22" t="s" s="2">
         <v>83</v>
@@ -4713,46 +4752,44 @@
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
-        <v>83</v>
+        <v>257</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" t="s" s="2">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="G23" t="s" s="2">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="H23" t="s" s="2">
         <v>83</v>
       </c>
       <c r="I23" t="s" s="2">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="J23" t="s" s="2">
         <v>96</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>115</v>
+        <v>258</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>255</v>
+        <v>259</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="N23" t="s" s="2">
-        <v>257</v>
-      </c>
-      <c r="O23" t="s" s="2">
-        <v>258</v>
-      </c>
+        <v>261</v>
+      </c>
+      <c r="O23" s="2"/>
       <c r="P23" t="s" s="2">
         <v>83</v>
       </c>
@@ -4776,13 +4813,13 @@
         <v>83</v>
       </c>
       <c r="X23" t="s" s="2">
-        <v>187</v>
+        <v>83</v>
       </c>
       <c r="Y23" t="s" s="2">
-        <v>259</v>
+        <v>83</v>
       </c>
       <c r="Z23" t="s" s="2">
-        <v>260</v>
+        <v>83</v>
       </c>
       <c r="AA23" t="s" s="2">
         <v>83</v>
@@ -4800,13 +4837,13 @@
         <v>83</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="AG23" t="s" s="2">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="AH23" t="s" s="2">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="AI23" t="s" s="2">
         <v>83</v>
@@ -4818,10 +4855,10 @@
         <v>83</v>
       </c>
       <c r="AL23" t="s" s="2">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="AM23" t="s" s="2">
-        <v>262</v>
+        <v>83</v>
       </c>
       <c r="AN23" t="s" s="2">
         <v>263</v>
@@ -4830,7 +4867,7 @@
         <v>264</v>
       </c>
       <c r="AP23" t="s" s="2">
-        <v>265</v>
+        <v>83</v>
       </c>
       <c r="AQ23" t="s" s="2">
         <v>83</v>
@@ -4838,10 +4875,10 @@
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -4858,25 +4895,25 @@
         <v>83</v>
       </c>
       <c r="I24" t="s" s="2">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="J24" t="s" s="2">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="K24" t="s" s="2">
-        <v>193</v>
+        <v>115</v>
       </c>
       <c r="L24" t="s" s="2">
+        <v>266</v>
+      </c>
+      <c r="M24" t="s" s="2">
         <v>267</v>
       </c>
-      <c r="M24" t="s" s="2">
+      <c r="N24" t="s" s="2">
         <v>268</v>
       </c>
-      <c r="N24" t="s" s="2">
+      <c r="O24" t="s" s="2">
         <v>269</v>
-      </c>
-      <c r="O24" t="s" s="2">
-        <v>270</v>
       </c>
       <c r="P24" t="s" s="2">
         <v>83</v>
@@ -4901,9 +4938,11 @@
         <v>83</v>
       </c>
       <c r="X24" t="s" s="2">
-        <v>187</v>
-      </c>
-      <c r="Y24" s="2"/>
+        <v>192</v>
+      </c>
+      <c r="Y24" t="s" s="2">
+        <v>270</v>
+      </c>
       <c r="Z24" t="s" s="2">
         <v>271</v>
       </c>
@@ -4923,13 +4962,13 @@
         <v>83</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="AG24" t="s" s="2">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="AH24" t="s" s="2">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="AI24" t="s" s="2">
         <v>83</v>
@@ -4938,22 +4977,22 @@
         <v>107</v>
       </c>
       <c r="AK24" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AL24" t="s" s="2">
         <v>272</v>
       </c>
-      <c r="AL24" t="s" s="2">
-        <v>83</v>
-      </c>
       <c r="AM24" t="s" s="2">
-        <v>83</v>
+        <v>273</v>
       </c>
       <c r="AN24" t="s" s="2">
-        <v>83</v>
+        <v>274</v>
       </c>
       <c r="AO24" t="s" s="2">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="AP24" t="s" s="2">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="AQ24" t="s" s="2">
         <v>83</v>
@@ -4961,14 +5000,14 @@
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
-        <v>276</v>
+        <v>83</v>
       </c>
       <c r="E25" s="2"/>
       <c r="F25" t="s" s="2">
@@ -4984,22 +5023,22 @@
         <v>83</v>
       </c>
       <c r="J25" t="s" s="2">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>278</v>
+        <v>279</v>
       </c>
       <c r="N25" t="s" s="2">
-        <v>279</v>
+        <v>280</v>
       </c>
       <c r="O25" t="s" s="2">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="P25" t="s" s="2">
         <v>83</v>
@@ -5009,7 +5048,7 @@
         <v>83</v>
       </c>
       <c r="S25" t="s" s="2">
-        <v>281</v>
+        <v>83</v>
       </c>
       <c r="T25" t="s" s="2">
         <v>83</v>
@@ -5024,14 +5063,12 @@
         <v>83</v>
       </c>
       <c r="X25" t="s" s="2">
+        <v>192</v>
+      </c>
+      <c r="Y25" s="2"/>
+      <c r="Z25" t="s" s="2">
         <v>282</v>
       </c>
-      <c r="Y25" t="s" s="2">
-        <v>283</v>
-      </c>
-      <c r="Z25" t="s" s="2">
-        <v>284</v>
-      </c>
       <c r="AA25" t="s" s="2">
         <v>83</v>
       </c>
@@ -5048,13 +5085,13 @@
         <v>83</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="AG25" t="s" s="2">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="AH25" t="s" s="2">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="AI25" t="s" s="2">
         <v>83</v>
@@ -5063,37 +5100,37 @@
         <v>107</v>
       </c>
       <c r="AK25" t="s" s="2">
-        <v>83</v>
+        <v>283</v>
       </c>
       <c r="AL25" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AM25" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AN25" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AO25" t="s" s="2">
+        <v>284</v>
+      </c>
+      <c r="AP25" t="s" s="2">
         <v>285</v>
       </c>
-      <c r="AM25" t="s" s="2">
-        <v>286</v>
-      </c>
-      <c r="AN25" t="s" s="2">
-        <v>287</v>
-      </c>
-      <c r="AO25" t="s" s="2">
-        <v>288</v>
-      </c>
-      <c r="AP25" t="s" s="2">
-        <v>289</v>
-      </c>
       <c r="AQ25" t="s" s="2">
-        <v>290</v>
+        <v>83</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
-        <v>83</v>
+        <v>287</v>
       </c>
       <c r="E26" s="2"/>
       <c r="F26" t="s" s="2">
@@ -5112,19 +5149,19 @@
         <v>96</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>292</v>
+        <v>199</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>293</v>
+        <v>288</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>294</v>
+        <v>289</v>
       </c>
       <c r="N26" t="s" s="2">
-        <v>295</v>
+        <v>290</v>
       </c>
       <c r="O26" t="s" s="2">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="P26" t="s" s="2">
         <v>83</v>
@@ -5134,7 +5171,7 @@
         <v>83</v>
       </c>
       <c r="S26" t="s" s="2">
-        <v>83</v>
+        <v>292</v>
       </c>
       <c r="T26" t="s" s="2">
         <v>83</v>
@@ -5149,13 +5186,13 @@
         <v>83</v>
       </c>
       <c r="X26" t="s" s="2">
-        <v>83</v>
+        <v>293</v>
       </c>
       <c r="Y26" t="s" s="2">
-        <v>83</v>
+        <v>294</v>
       </c>
       <c r="Z26" t="s" s="2">
-        <v>83</v>
+        <v>295</v>
       </c>
       <c r="AA26" t="s" s="2">
         <v>83</v>
@@ -5173,10 +5210,10 @@
         <v>83</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="AG26" t="s" s="2">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="AH26" t="s" s="2">
         <v>95</v>
@@ -5188,25 +5225,25 @@
         <v>107</v>
       </c>
       <c r="AK26" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AL26" t="s" s="2">
+        <v>296</v>
+      </c>
+      <c r="AM26" t="s" s="2">
         <v>297</v>
       </c>
-      <c r="AL26" t="s" s="2">
+      <c r="AN26" t="s" s="2">
         <v>298</v>
       </c>
-      <c r="AM26" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AN26" t="s" s="2">
+      <c r="AO26" t="s" s="2">
         <v>299</v>
       </c>
-      <c r="AO26" t="s" s="2">
+      <c r="AP26" t="s" s="2">
         <v>300</v>
       </c>
-      <c r="AP26" t="s" s="2">
+      <c r="AQ26" t="s" s="2">
         <v>301</v>
-      </c>
-      <c r="AQ26" t="s" s="2">
-        <v>83</v>
       </c>
     </row>
     <row r="27">
@@ -5222,10 +5259,10 @@
       </c>
       <c r="E27" s="2"/>
       <c r="F27" t="s" s="2">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="G27" t="s" s="2">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="H27" t="s" s="2">
         <v>83</v>
@@ -5248,7 +5285,9 @@
       <c r="N27" t="s" s="2">
         <v>306</v>
       </c>
-      <c r="O27" s="2"/>
+      <c r="O27" t="s" s="2">
+        <v>307</v>
+      </c>
       <c r="P27" t="s" s="2">
         <v>83</v>
       </c>
@@ -5302,7 +5341,7 @@
         <v>81</v>
       </c>
       <c r="AH27" t="s" s="2">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="AI27" t="s" s="2">
         <v>83</v>
@@ -5311,22 +5350,22 @@
         <v>107</v>
       </c>
       <c r="AK27" t="s" s="2">
-        <v>83</v>
+        <v>308</v>
       </c>
       <c r="AL27" t="s" s="2">
-        <v>83</v>
+        <v>309</v>
       </c>
       <c r="AM27" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AN27" t="s" s="2">
-        <v>287</v>
+        <v>310</v>
       </c>
       <c r="AO27" t="s" s="2">
-        <v>307</v>
+        <v>311</v>
       </c>
       <c r="AP27" t="s" s="2">
-        <v>301</v>
+        <v>312</v>
       </c>
       <c r="AQ27" t="s" s="2">
         <v>83</v>
@@ -5334,21 +5373,21 @@
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
-        <v>309</v>
+        <v>83</v>
       </c>
       <c r="E28" s="2"/>
       <c r="F28" t="s" s="2">
         <v>81</v>
       </c>
       <c r="G28" t="s" s="2">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="H28" t="s" s="2">
         <v>83</v>
@@ -5360,20 +5399,18 @@
         <v>96</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>310</v>
+        <v>314</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>311</v>
+        <v>315</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>312</v>
+        <v>316</v>
       </c>
       <c r="N28" t="s" s="2">
-        <v>313</v>
-      </c>
-      <c r="O28" t="s" s="2">
-        <v>314</v>
-      </c>
+        <v>317</v>
+      </c>
+      <c r="O28" s="2"/>
       <c r="P28" t="s" s="2">
         <v>83</v>
       </c>
@@ -5421,13 +5458,13 @@
         <v>83</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>308</v>
+        <v>313</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH28" t="s" s="2">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="AI28" t="s" s="2">
         <v>83</v>
@@ -5439,19 +5476,19 @@
         <v>83</v>
       </c>
       <c r="AL28" t="s" s="2">
-        <v>315</v>
+        <v>83</v>
       </c>
       <c r="AM28" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AN28" t="s" s="2">
-        <v>316</v>
+        <v>298</v>
       </c>
       <c r="AO28" t="s" s="2">
-        <v>317</v>
+        <v>318</v>
       </c>
       <c r="AP28" t="s" s="2">
-        <v>318</v>
+        <v>312</v>
       </c>
       <c r="AQ28" t="s" s="2">
         <v>83</v>
@@ -5470,7 +5507,7 @@
       </c>
       <c r="E29" s="2"/>
       <c r="F29" t="s" s="2">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="G29" t="s" s="2">
         <v>95</v>
@@ -5534,14 +5571,16 @@
         <v>83</v>
       </c>
       <c r="AB29" t="s" s="2">
-        <v>326</v>
-      </c>
-      <c r="AC29" s="2"/>
+        <v>83</v>
+      </c>
+      <c r="AC29" t="s" s="2">
+        <v>83</v>
+      </c>
       <c r="AD29" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AE29" t="s" s="2">
-        <v>327</v>
+        <v>83</v>
       </c>
       <c r="AF29" t="s" s="2">
         <v>319</v>
@@ -5562,19 +5601,19 @@
         <v>83</v>
       </c>
       <c r="AL29" t="s" s="2">
+        <v>326</v>
+      </c>
+      <c r="AM29" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AN29" t="s" s="2">
+        <v>327</v>
+      </c>
+      <c r="AO29" t="s" s="2">
         <v>328</v>
       </c>
-      <c r="AM29" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AN29" t="s" s="2">
+      <c r="AP29" t="s" s="2">
         <v>329</v>
-      </c>
-      <c r="AO29" t="s" s="2">
-        <v>330</v>
-      </c>
-      <c r="AP29" t="s" s="2">
-        <v>331</v>
       </c>
       <c r="AQ29" t="s" s="2">
         <v>83</v>
@@ -5582,16 +5621,14 @@
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>319</v>
-      </c>
-      <c r="C30" t="s" s="2">
-        <v>333</v>
-      </c>
+        <v>330</v>
+      </c>
+      <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
-        <v>320</v>
+        <v>331</v>
       </c>
       <c r="E30" s="2"/>
       <c r="F30" t="s" s="2">
@@ -5610,19 +5647,19 @@
         <v>96</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>321</v>
+        <v>332</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>322</v>
+        <v>333</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>323</v>
+        <v>334</v>
       </c>
       <c r="N30" t="s" s="2">
-        <v>324</v>
+        <v>335</v>
       </c>
       <c r="O30" t="s" s="2">
-        <v>325</v>
+        <v>336</v>
       </c>
       <c r="P30" t="s" s="2">
         <v>83</v>
@@ -5659,19 +5696,17 @@
         <v>83</v>
       </c>
       <c r="AB30" t="s" s="2">
-        <v>83</v>
-      </c>
-      <c r="AC30" t="s" s="2">
-        <v>83</v>
-      </c>
+        <v>337</v>
+      </c>
+      <c r="AC30" s="2"/>
       <c r="AD30" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AE30" t="s" s="2">
-        <v>83</v>
+        <v>338</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>319</v>
+        <v>330</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>81</v>
@@ -5686,22 +5721,22 @@
         <v>107</v>
       </c>
       <c r="AK30" t="s" s="2">
-        <v>334</v>
+        <v>83</v>
       </c>
       <c r="AL30" t="s" s="2">
-        <v>328</v>
+        <v>339</v>
       </c>
       <c r="AM30" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AN30" t="s" s="2">
-        <v>329</v>
+        <v>340</v>
       </c>
       <c r="AO30" t="s" s="2">
-        <v>330</v>
+        <v>341</v>
       </c>
       <c r="AP30" t="s" s="2">
-        <v>331</v>
+        <v>342</v>
       </c>
       <c r="AQ30" t="s" s="2">
         <v>83</v>
@@ -5709,18 +5744,20 @@
     </row>
     <row r="31">
       <c r="A31" t="s" s="2">
-        <v>335</v>
+        <v>343</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>335</v>
-      </c>
-      <c r="C31" s="2"/>
+        <v>330</v>
+      </c>
+      <c r="C31" t="s" s="2">
+        <v>344</v>
+      </c>
       <c r="D31" t="s" s="2">
-        <v>83</v>
+        <v>331</v>
       </c>
       <c r="E31" s="2"/>
       <c r="F31" t="s" s="2">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="G31" t="s" s="2">
         <v>95</v>
@@ -5735,18 +5772,20 @@
         <v>96</v>
       </c>
       <c r="K31" t="s" s="2">
+        <v>332</v>
+      </c>
+      <c r="L31" t="s" s="2">
+        <v>333</v>
+      </c>
+      <c r="M31" t="s" s="2">
+        <v>334</v>
+      </c>
+      <c r="N31" t="s" s="2">
+        <v>335</v>
+      </c>
+      <c r="O31" t="s" s="2">
         <v>336</v>
       </c>
-      <c r="L31" t="s" s="2">
-        <v>337</v>
-      </c>
-      <c r="M31" t="s" s="2">
-        <v>338</v>
-      </c>
-      <c r="N31" t="s" s="2">
-        <v>339</v>
-      </c>
-      <c r="O31" s="2"/>
       <c r="P31" t="s" s="2">
         <v>83</v>
       </c>
@@ -5794,7 +5833,7 @@
         <v>83</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>335</v>
+        <v>330</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>81</v>
@@ -5809,10 +5848,10 @@
         <v>107</v>
       </c>
       <c r="AK31" t="s" s="2">
-        <v>83</v>
+        <v>345</v>
       </c>
       <c r="AL31" t="s" s="2">
-        <v>83</v>
+        <v>339</v>
       </c>
       <c r="AM31" t="s" s="2">
         <v>83</v>
@@ -5832,10 +5871,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s" s="2">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -5846,7 +5885,7 @@
         <v>81</v>
       </c>
       <c r="G32" t="s" s="2">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="H32" t="s" s="2">
         <v>83</v>
@@ -5858,18 +5897,18 @@
         <v>96</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>346</v>
-      </c>
-      <c r="N32" s="2"/>
-      <c r="O32" t="s" s="2">
-        <v>347</v>
-      </c>
+        <v>349</v>
+      </c>
+      <c r="N32" t="s" s="2">
+        <v>350</v>
+      </c>
+      <c r="O32" s="2"/>
       <c r="P32" t="s" s="2">
         <v>83</v>
       </c>
@@ -5917,13 +5956,13 @@
         <v>83</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH32" t="s" s="2">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="AI32" t="s" s="2">
         <v>83</v>
@@ -5935,19 +5974,19 @@
         <v>83</v>
       </c>
       <c r="AL32" t="s" s="2">
-        <v>348</v>
+        <v>83</v>
       </c>
       <c r="AM32" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AN32" t="s" s="2">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="AO32" t="s" s="2">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="AP32" t="s" s="2">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="AQ32" t="s" s="2">
         <v>83</v>
@@ -5955,10 +5994,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s" s="2">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -5969,7 +6008,7 @@
         <v>81</v>
       </c>
       <c r="G33" t="s" s="2">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="H33" t="s" s="2">
         <v>83</v>
@@ -5981,19 +6020,17 @@
         <v>96</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>355</v>
-      </c>
-      <c r="N33" t="s" s="2">
-        <v>356</v>
-      </c>
+        <v>357</v>
+      </c>
+      <c r="N33" s="2"/>
       <c r="O33" t="s" s="2">
-        <v>357</v>
+        <v>358</v>
       </c>
       <c r="P33" t="s" s="2">
         <v>83</v>
@@ -6042,16 +6079,16 @@
         <v>83</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH33" t="s" s="2">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="AI33" t="s" s="2">
-        <v>358</v>
+        <v>83</v>
       </c>
       <c r="AJ33" t="s" s="2">
         <v>107</v>
@@ -6060,10 +6097,10 @@
         <v>83</v>
       </c>
       <c r="AL33" t="s" s="2">
-        <v>83</v>
+        <v>359</v>
       </c>
       <c r="AM33" t="s" s="2">
-        <v>359</v>
+        <v>83</v>
       </c>
       <c r="AN33" t="s" s="2">
         <v>360</v>
@@ -6072,10 +6109,10 @@
         <v>361</v>
       </c>
       <c r="AP33" t="s" s="2">
-        <v>83</v>
+        <v>362</v>
       </c>
       <c r="AQ33" t="s" s="2">
-        <v>362</v>
+        <v>83</v>
       </c>
     </row>
     <row r="34">
@@ -6103,22 +6140,22 @@
         <v>83</v>
       </c>
       <c r="J34" t="s" s="2">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>193</v>
+        <v>364</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>364</v>
+        <v>365</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>365</v>
+        <v>366</v>
       </c>
       <c r="N34" t="s" s="2">
-        <v>366</v>
+        <v>367</v>
       </c>
       <c r="O34" t="s" s="2">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="P34" t="s" s="2">
         <v>83</v>
@@ -6143,13 +6180,13 @@
         <v>83</v>
       </c>
       <c r="X34" t="s" s="2">
-        <v>198</v>
+        <v>83</v>
       </c>
       <c r="Y34" t="s" s="2">
-        <v>368</v>
+        <v>83</v>
       </c>
       <c r="Z34" t="s" s="2">
-        <v>369</v>
+        <v>83</v>
       </c>
       <c r="AA34" t="s" s="2">
         <v>83</v>
@@ -6176,7 +6213,7 @@
         <v>95</v>
       </c>
       <c r="AI34" t="s" s="2">
-        <v>370</v>
+        <v>369</v>
       </c>
       <c r="AJ34" t="s" s="2">
         <v>107</v>
@@ -6188,38 +6225,38 @@
         <v>83</v>
       </c>
       <c r="AM34" t="s" s="2">
-        <v>83</v>
+        <v>370</v>
       </c>
       <c r="AN34" t="s" s="2">
-        <v>138</v>
+        <v>371</v>
       </c>
       <c r="AO34" t="s" s="2">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="AP34" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AQ34" t="s" s="2">
-        <v>83</v>
+        <v>373</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
-        <v>373</v>
+        <v>83</v>
       </c>
       <c r="E35" s="2"/>
       <c r="F35" t="s" s="2">
         <v>81</v>
       </c>
       <c r="G35" t="s" s="2">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="H35" t="s" s="2">
         <v>83</v>
@@ -6231,19 +6268,19 @@
         <v>83</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>374</v>
+        <v>375</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>375</v>
+        <v>376</v>
       </c>
       <c r="N35" t="s" s="2">
-        <v>376</v>
+        <v>377</v>
       </c>
       <c r="O35" t="s" s="2">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="P35" t="s" s="2">
         <v>83</v>
@@ -6268,13 +6305,13 @@
         <v>83</v>
       </c>
       <c r="X35" t="s" s="2">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="Y35" t="s" s="2">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="Z35" t="s" s="2">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="AA35" t="s" s="2">
         <v>83</v>
@@ -6292,16 +6329,16 @@
         <v>83</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH35" t="s" s="2">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="AI35" t="s" s="2">
-        <v>83</v>
+        <v>381</v>
       </c>
       <c r="AJ35" t="s" s="2">
         <v>107</v>
@@ -6313,10 +6350,10 @@
         <v>83</v>
       </c>
       <c r="AM35" t="s" s="2">
-        <v>380</v>
+        <v>83</v>
       </c>
       <c r="AN35" t="s" s="2">
-        <v>381</v>
+        <v>138</v>
       </c>
       <c r="AO35" t="s" s="2">
         <v>382</v>
@@ -6325,19 +6362,19 @@
         <v>83</v>
       </c>
       <c r="AQ35" t="s" s="2">
-        <v>383</v>
+        <v>83</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
-        <v>83</v>
+        <v>384</v>
       </c>
       <c r="E36" s="2"/>
       <c r="F36" t="s" s="2">
@@ -6356,19 +6393,19 @@
         <v>83</v>
       </c>
       <c r="K36" t="s" s="2">
+        <v>199</v>
+      </c>
+      <c r="L36" t="s" s="2">
         <v>385</v>
       </c>
-      <c r="L36" t="s" s="2">
+      <c r="M36" t="s" s="2">
         <v>386</v>
       </c>
-      <c r="M36" t="s" s="2">
+      <c r="N36" t="s" s="2">
         <v>387</v>
       </c>
-      <c r="N36" t="s" s="2">
+      <c r="O36" t="s" s="2">
         <v>388</v>
-      </c>
-      <c r="O36" t="s" s="2">
-        <v>389</v>
       </c>
       <c r="P36" t="s" s="2">
         <v>83</v>
@@ -6393,13 +6430,13 @@
         <v>83</v>
       </c>
       <c r="X36" t="s" s="2">
-        <v>83</v>
+        <v>205</v>
       </c>
       <c r="Y36" t="s" s="2">
-        <v>83</v>
+        <v>389</v>
       </c>
       <c r="Z36" t="s" s="2">
-        <v>83</v>
+        <v>390</v>
       </c>
       <c r="AA36" t="s" s="2">
         <v>83</v>
@@ -6417,7 +6454,7 @@
         <v>83</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>384</v>
+        <v>383</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>81</v>
@@ -6438,27 +6475,27 @@
         <v>83</v>
       </c>
       <c r="AM36" t="s" s="2">
-        <v>83</v>
+        <v>391</v>
       </c>
       <c r="AN36" t="s" s="2">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="AO36" t="s" s="2">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="AP36" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AQ36" t="s" s="2">
-        <v>83</v>
+        <v>394</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="2">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -6469,7 +6506,7 @@
         <v>81</v>
       </c>
       <c r="G37" t="s" s="2">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="H37" t="s" s="2">
         <v>83</v>
@@ -6481,18 +6518,20 @@
         <v>83</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>193</v>
+        <v>396</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>393</v>
+        <v>397</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>394</v>
+        <v>398</v>
       </c>
       <c r="N37" t="s" s="2">
-        <v>395</v>
-      </c>
-      <c r="O37" s="2"/>
+        <v>399</v>
+      </c>
+      <c r="O37" t="s" s="2">
+        <v>400</v>
+      </c>
       <c r="P37" t="s" s="2">
         <v>83</v>
       </c>
@@ -6516,13 +6555,13 @@
         <v>83</v>
       </c>
       <c r="X37" t="s" s="2">
-        <v>282</v>
+        <v>83</v>
       </c>
       <c r="Y37" t="s" s="2">
-        <v>396</v>
+        <v>83</v>
       </c>
       <c r="Z37" t="s" s="2">
-        <v>397</v>
+        <v>83</v>
       </c>
       <c r="AA37" t="s" s="2">
         <v>83</v>
@@ -6540,13 +6579,13 @@
         <v>83</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH37" t="s" s="2">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="AI37" t="s" s="2">
         <v>83</v>
@@ -6561,27 +6600,27 @@
         <v>83</v>
       </c>
       <c r="AM37" t="s" s="2">
-        <v>398</v>
+        <v>83</v>
       </c>
       <c r="AN37" t="s" s="2">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="AO37" t="s" s="2">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="AP37" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AQ37" t="s" s="2">
-        <v>401</v>
+        <v>83</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="s" s="2">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -6604,20 +6643,18 @@
         <v>83</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>403</v>
+        <v>404</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>404</v>
+        <v>405</v>
       </c>
       <c r="N38" t="s" s="2">
-        <v>405</v>
-      </c>
-      <c r="O38" t="s" s="2">
         <v>406</v>
       </c>
+      <c r="O38" s="2"/>
       <c r="P38" t="s" s="2">
         <v>83</v>
       </c>
@@ -6641,7 +6678,7 @@
         <v>83</v>
       </c>
       <c r="X38" t="s" s="2">
-        <v>282</v>
+        <v>293</v>
       </c>
       <c r="Y38" t="s" s="2">
         <v>407</v>
@@ -6665,7 +6702,7 @@
         <v>83</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>402</v>
+        <v>403</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>81</v>
@@ -6686,27 +6723,27 @@
         <v>83</v>
       </c>
       <c r="AM38" t="s" s="2">
-        <v>83</v>
+        <v>409</v>
       </c>
       <c r="AN38" t="s" s="2">
-        <v>409</v>
+        <v>410</v>
       </c>
       <c r="AO38" t="s" s="2">
-        <v>410</v>
+        <v>411</v>
       </c>
       <c r="AP38" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AQ38" t="s" s="2">
-        <v>83</v>
+        <v>412</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="2">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -6729,18 +6766,20 @@
         <v>83</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>412</v>
+        <v>199</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>413</v>
+        <v>414</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>414</v>
+        <v>415</v>
       </c>
       <c r="N39" t="s" s="2">
-        <v>415</v>
-      </c>
-      <c r="O39" s="2"/>
+        <v>416</v>
+      </c>
+      <c r="O39" t="s" s="2">
+        <v>417</v>
+      </c>
       <c r="P39" t="s" s="2">
         <v>83</v>
       </c>
@@ -6764,13 +6803,13 @@
         <v>83</v>
       </c>
       <c r="X39" t="s" s="2">
-        <v>83</v>
+        <v>293</v>
       </c>
       <c r="Y39" t="s" s="2">
-        <v>83</v>
+        <v>418</v>
       </c>
       <c r="Z39" t="s" s="2">
-        <v>83</v>
+        <v>419</v>
       </c>
       <c r="AA39" t="s" s="2">
         <v>83</v>
@@ -6788,7 +6827,7 @@
         <v>83</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>81</v>
@@ -6809,27 +6848,27 @@
         <v>83</v>
       </c>
       <c r="AM39" t="s" s="2">
-        <v>416</v>
+        <v>83</v>
       </c>
       <c r="AN39" t="s" s="2">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="AO39" t="s" s="2">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="AP39" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AQ39" t="s" s="2">
-        <v>419</v>
+        <v>83</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="s" s="2">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -6852,16 +6891,16 @@
         <v>83</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="N40" t="s" s="2">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="O40" s="2"/>
       <c r="P40" t="s" s="2">
@@ -6911,7 +6950,7 @@
         <v>83</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>81</v>
@@ -6932,27 +6971,27 @@
         <v>83</v>
       </c>
       <c r="AM40" t="s" s="2">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="AN40" t="s" s="2">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="AO40" t="s" s="2">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="AP40" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AQ40" t="s" s="2">
-        <v>428</v>
+        <v>430</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -6963,7 +7002,7 @@
         <v>81</v>
       </c>
       <c r="G41" t="s" s="2">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="H41" t="s" s="2">
         <v>83</v>
@@ -6975,20 +7014,18 @@
         <v>83</v>
       </c>
       <c r="K41" t="s" s="2">
-        <v>430</v>
+        <v>432</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="N41" t="s" s="2">
-        <v>433</v>
-      </c>
-      <c r="O41" t="s" s="2">
-        <v>434</v>
-      </c>
+        <v>435</v>
+      </c>
+      <c r="O41" s="2"/>
       <c r="P41" t="s" s="2">
         <v>83</v>
       </c>
@@ -7036,19 +7073,19 @@
         <v>83</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH41" t="s" s="2">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="AI41" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AJ41" t="s" s="2">
-        <v>435</v>
+        <v>107</v>
       </c>
       <c r="AK41" t="s" s="2">
         <v>83</v>
@@ -7057,27 +7094,27 @@
         <v>83</v>
       </c>
       <c r="AM41" t="s" s="2">
-        <v>83</v>
+        <v>436</v>
       </c>
       <c r="AN41" t="s" s="2">
-        <v>436</v>
+        <v>437</v>
       </c>
       <c r="AO41" t="s" s="2">
-        <v>437</v>
+        <v>438</v>
       </c>
       <c r="AP41" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AQ41" t="s" s="2">
-        <v>83</v>
+        <v>439</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -7088,7 +7125,7 @@
         <v>81</v>
       </c>
       <c r="G42" t="s" s="2">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="H42" t="s" s="2">
         <v>83</v>
@@ -7100,16 +7137,20 @@
         <v>83</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>172</v>
+        <v>441</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>173</v>
+        <v>442</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>174</v>
-      </c>
-      <c r="N42" s="2"/>
-      <c r="O42" s="2"/>
+        <v>443</v>
+      </c>
+      <c r="N42" t="s" s="2">
+        <v>444</v>
+      </c>
+      <c r="O42" t="s" s="2">
+        <v>445</v>
+      </c>
       <c r="P42" t="s" s="2">
         <v>83</v>
       </c>
@@ -7157,19 +7198,19 @@
         <v>83</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>175</v>
+        <v>440</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH42" t="s" s="2">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="AI42" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AJ42" t="s" s="2">
-        <v>83</v>
+        <v>446</v>
       </c>
       <c r="AK42" t="s" s="2">
         <v>83</v>
@@ -7181,10 +7222,10 @@
         <v>83</v>
       </c>
       <c r="AN42" t="s" s="2">
-        <v>83</v>
+        <v>447</v>
       </c>
       <c r="AO42" t="s" s="2">
-        <v>176</v>
+        <v>448</v>
       </c>
       <c r="AP42" t="s" s="2">
         <v>83</v>
@@ -7195,21 +7236,21 @@
     </row>
     <row r="43">
       <c r="A43" t="s" s="2">
-        <v>439</v>
+        <v>449</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>439</v>
+        <v>449</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
-        <v>155</v>
+        <v>83</v>
       </c>
       <c r="E43" s="2"/>
       <c r="F43" t="s" s="2">
         <v>81</v>
       </c>
       <c r="G43" t="s" s="2">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="H43" t="s" s="2">
         <v>83</v>
@@ -7221,17 +7262,15 @@
         <v>83</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>140</v>
+        <v>175</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>179</v>
-      </c>
-      <c r="N43" t="s" s="2">
-        <v>158</v>
-      </c>
+        <v>177</v>
+      </c>
+      <c r="N43" s="2"/>
       <c r="O43" s="2"/>
       <c r="P43" t="s" s="2">
         <v>83</v>
@@ -7280,19 +7319,19 @@
         <v>83</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH43" t="s" s="2">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="AI43" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AJ43" t="s" s="2">
-        <v>146</v>
+        <v>83</v>
       </c>
       <c r="AK43" t="s" s="2">
         <v>83</v>
@@ -7307,7 +7346,7 @@
         <v>83</v>
       </c>
       <c r="AO43" t="s" s="2">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="AP43" t="s" s="2">
         <v>83</v>
@@ -7318,14 +7357,14 @@
     </row>
     <row r="44">
       <c r="A44" t="s" s="2">
-        <v>440</v>
+        <v>450</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>440</v>
+        <v>450</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
-        <v>441</v>
+        <v>155</v>
       </c>
       <c r="E44" s="2"/>
       <c r="F44" t="s" s="2">
@@ -7338,26 +7377,24 @@
         <v>83</v>
       </c>
       <c r="I44" t="s" s="2">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="J44" t="s" s="2">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="K44" t="s" s="2">
         <v>140</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>442</v>
+        <v>182</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>443</v>
+        <v>183</v>
       </c>
       <c r="N44" t="s" s="2">
         <v>158</v>
       </c>
-      <c r="O44" t="s" s="2">
-        <v>159</v>
-      </c>
+      <c r="O44" s="2"/>
       <c r="P44" t="s" s="2">
         <v>83</v>
       </c>
@@ -7405,7 +7442,7 @@
         <v>83</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>444</v>
+        <v>185</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>81</v>
@@ -7432,7 +7469,7 @@
         <v>83</v>
       </c>
       <c r="AO44" t="s" s="2">
-        <v>138</v>
+        <v>179</v>
       </c>
       <c r="AP44" t="s" s="2">
         <v>83</v>
@@ -7443,42 +7480,46 @@
     </row>
     <row r="45">
       <c r="A45" t="s" s="2">
-        <v>445</v>
+        <v>451</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>445</v>
+        <v>451</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
-        <v>83</v>
+        <v>452</v>
       </c>
       <c r="E45" s="2"/>
       <c r="F45" t="s" s="2">
         <v>81</v>
       </c>
       <c r="G45" t="s" s="2">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="H45" t="s" s="2">
         <v>83</v>
       </c>
       <c r="I45" t="s" s="2">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="J45" t="s" s="2">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="K45" t="s" s="2">
-        <v>446</v>
+        <v>140</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>447</v>
+        <v>453</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>448</v>
-      </c>
-      <c r="N45" s="2"/>
-      <c r="O45" s="2"/>
+        <v>454</v>
+      </c>
+      <c r="N45" t="s" s="2">
+        <v>158</v>
+      </c>
+      <c r="O45" t="s" s="2">
+        <v>159</v>
+      </c>
       <c r="P45" t="s" s="2">
         <v>83</v>
       </c>
@@ -7526,19 +7567,19 @@
         <v>83</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>445</v>
+        <v>455</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH45" t="s" s="2">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="AI45" t="s" s="2">
-        <v>449</v>
+        <v>83</v>
       </c>
       <c r="AJ45" t="s" s="2">
-        <v>107</v>
+        <v>146</v>
       </c>
       <c r="AK45" t="s" s="2">
         <v>83</v>
@@ -7550,10 +7591,10 @@
         <v>83</v>
       </c>
       <c r="AN45" t="s" s="2">
-        <v>450</v>
+        <v>83</v>
       </c>
       <c r="AO45" t="s" s="2">
-        <v>451</v>
+        <v>138</v>
       </c>
       <c r="AP45" t="s" s="2">
         <v>83</v>
@@ -7564,10 +7605,10 @@
     </row>
     <row r="46">
       <c r="A46" t="s" s="2">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -7590,13 +7631,13 @@
         <v>83</v>
       </c>
       <c r="K46" t="s" s="2">
-        <v>446</v>
+        <v>457</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>453</v>
+        <v>458</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>454</v>
+        <v>459</v>
       </c>
       <c r="N46" s="2"/>
       <c r="O46" s="2"/>
@@ -7647,7 +7688,7 @@
         <v>83</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>452</v>
+        <v>456</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>81</v>
@@ -7656,7 +7697,7 @@
         <v>95</v>
       </c>
       <c r="AI46" t="s" s="2">
-        <v>449</v>
+        <v>460</v>
       </c>
       <c r="AJ46" t="s" s="2">
         <v>107</v>
@@ -7671,10 +7712,10 @@
         <v>83</v>
       </c>
       <c r="AN46" t="s" s="2">
-        <v>450</v>
+        <v>461</v>
       </c>
       <c r="AO46" t="s" s="2">
-        <v>455</v>
+        <v>462</v>
       </c>
       <c r="AP46" t="s" s="2">
         <v>83</v>
@@ -7685,10 +7726,10 @@
     </row>
     <row r="47">
       <c r="A47" t="s" s="2">
-        <v>456</v>
+        <v>463</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>456</v>
+        <v>463</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -7711,20 +7752,16 @@
         <v>83</v>
       </c>
       <c r="K47" t="s" s="2">
-        <v>193</v>
+        <v>457</v>
       </c>
       <c r="L47" t="s" s="2">
-        <v>457</v>
+        <v>464</v>
       </c>
       <c r="M47" t="s" s="2">
-        <v>458</v>
-      </c>
-      <c r="N47" t="s" s="2">
-        <v>459</v>
-      </c>
-      <c r="O47" t="s" s="2">
-        <v>460</v>
-      </c>
+        <v>465</v>
+      </c>
+      <c r="N47" s="2"/>
+      <c r="O47" s="2"/>
       <c r="P47" t="s" s="2">
         <v>83</v>
       </c>
@@ -7748,13 +7785,13 @@
         <v>83</v>
       </c>
       <c r="X47" t="s" s="2">
-        <v>119</v>
+        <v>83</v>
       </c>
       <c r="Y47" t="s" s="2">
-        <v>461</v>
+        <v>83</v>
       </c>
       <c r="Z47" t="s" s="2">
-        <v>462</v>
+        <v>83</v>
       </c>
       <c r="AA47" t="s" s="2">
         <v>83</v>
@@ -7772,7 +7809,7 @@
         <v>83</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>456</v>
+        <v>463</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>81</v>
@@ -7781,7 +7818,7 @@
         <v>95</v>
       </c>
       <c r="AI47" t="s" s="2">
-        <v>83</v>
+        <v>460</v>
       </c>
       <c r="AJ47" t="s" s="2">
         <v>107</v>
@@ -7793,13 +7830,13 @@
         <v>83</v>
       </c>
       <c r="AM47" t="s" s="2">
-        <v>463</v>
+        <v>83</v>
       </c>
       <c r="AN47" t="s" s="2">
-        <v>464</v>
+        <v>461</v>
       </c>
       <c r="AO47" t="s" s="2">
-        <v>382</v>
+        <v>466</v>
       </c>
       <c r="AP47" t="s" s="2">
         <v>83</v>
@@ -7810,10 +7847,10 @@
     </row>
     <row r="48">
       <c r="A48" t="s" s="2">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -7824,7 +7861,7 @@
         <v>81</v>
       </c>
       <c r="G48" t="s" s="2">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="H48" t="s" s="2">
         <v>83</v>
@@ -7836,19 +7873,19 @@
         <v>83</v>
       </c>
       <c r="K48" t="s" s="2">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="L48" t="s" s="2">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="M48" t="s" s="2">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="N48" t="s" s="2">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="O48" t="s" s="2">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="P48" t="s" s="2">
         <v>83</v>
@@ -7873,13 +7910,13 @@
         <v>83</v>
       </c>
       <c r="X48" t="s" s="2">
-        <v>282</v>
+        <v>119</v>
       </c>
       <c r="Y48" t="s" s="2">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="Z48" t="s" s="2">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="AA48" t="s" s="2">
         <v>83</v>
@@ -7897,13 +7934,13 @@
         <v>83</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="AG48" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH48" t="s" s="2">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="AI48" t="s" s="2">
         <v>83</v>
@@ -7918,13 +7955,13 @@
         <v>83</v>
       </c>
       <c r="AM48" t="s" s="2">
-        <v>463</v>
+        <v>474</v>
       </c>
       <c r="AN48" t="s" s="2">
-        <v>464</v>
+        <v>475</v>
       </c>
       <c r="AO48" t="s" s="2">
-        <v>382</v>
+        <v>393</v>
       </c>
       <c r="AP48" t="s" s="2">
         <v>83</v>
@@ -7935,10 +7972,10 @@
     </row>
     <row r="49">
       <c r="A49" t="s" s="2">
-        <v>472</v>
+        <v>476</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>472</v>
+        <v>476</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -7949,7 +7986,7 @@
         <v>81</v>
       </c>
       <c r="G49" t="s" s="2">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="H49" t="s" s="2">
         <v>83</v>
@@ -7961,17 +7998,19 @@
         <v>83</v>
       </c>
       <c r="K49" t="s" s="2">
-        <v>473</v>
+        <v>199</v>
       </c>
       <c r="L49" t="s" s="2">
-        <v>474</v>
+        <v>477</v>
       </c>
       <c r="M49" t="s" s="2">
-        <v>475</v>
-      </c>
-      <c r="N49" s="2"/>
+        <v>478</v>
+      </c>
+      <c r="N49" t="s" s="2">
+        <v>479</v>
+      </c>
       <c r="O49" t="s" s="2">
-        <v>476</v>
+        <v>480</v>
       </c>
       <c r="P49" t="s" s="2">
         <v>83</v>
@@ -7996,13 +8035,13 @@
         <v>83</v>
       </c>
       <c r="X49" t="s" s="2">
-        <v>83</v>
+        <v>293</v>
       </c>
       <c r="Y49" t="s" s="2">
-        <v>83</v>
+        <v>481</v>
       </c>
       <c r="Z49" t="s" s="2">
-        <v>83</v>
+        <v>482</v>
       </c>
       <c r="AA49" t="s" s="2">
         <v>83</v>
@@ -8020,13 +8059,13 @@
         <v>83</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>472</v>
+        <v>476</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH49" t="s" s="2">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="AI49" t="s" s="2">
         <v>83</v>
@@ -8041,13 +8080,13 @@
         <v>83</v>
       </c>
       <c r="AM49" t="s" s="2">
-        <v>83</v>
+        <v>474</v>
       </c>
       <c r="AN49" t="s" s="2">
-        <v>83</v>
+        <v>475</v>
       </c>
       <c r="AO49" t="s" s="2">
-        <v>477</v>
+        <v>393</v>
       </c>
       <c r="AP49" t="s" s="2">
         <v>83</v>
@@ -8058,10 +8097,10 @@
     </row>
     <row r="50">
       <c r="A50" t="s" s="2">
-        <v>478</v>
+        <v>483</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>478</v>
+        <v>483</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -8084,16 +8123,18 @@
         <v>83</v>
       </c>
       <c r="K50" t="s" s="2">
-        <v>172</v>
+        <v>484</v>
       </c>
       <c r="L50" t="s" s="2">
-        <v>479</v>
+        <v>485</v>
       </c>
       <c r="M50" t="s" s="2">
-        <v>480</v>
+        <v>486</v>
       </c>
       <c r="N50" s="2"/>
-      <c r="O50" s="2"/>
+      <c r="O50" t="s" s="2">
+        <v>487</v>
+      </c>
       <c r="P50" t="s" s="2">
         <v>83</v>
       </c>
@@ -8141,7 +8182,7 @@
         <v>83</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>478</v>
+        <v>483</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>81</v>
@@ -8165,10 +8206,10 @@
         <v>83</v>
       </c>
       <c r="AN50" t="s" s="2">
-        <v>450</v>
+        <v>83</v>
       </c>
       <c r="AO50" t="s" s="2">
-        <v>481</v>
+        <v>488</v>
       </c>
       <c r="AP50" t="s" s="2">
         <v>83</v>
@@ -8179,10 +8220,10 @@
     </row>
     <row r="51">
       <c r="A51" t="s" s="2">
-        <v>482</v>
+        <v>489</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>482</v>
+        <v>489</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -8193,7 +8234,7 @@
         <v>81</v>
       </c>
       <c r="G51" t="s" s="2">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="H51" t="s" s="2">
         <v>83</v>
@@ -8202,20 +8243,18 @@
         <v>83</v>
       </c>
       <c r="J51" t="s" s="2">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="K51" t="s" s="2">
-        <v>483</v>
+        <v>175</v>
       </c>
       <c r="L51" t="s" s="2">
-        <v>484</v>
+        <v>490</v>
       </c>
       <c r="M51" t="s" s="2">
-        <v>485</v>
-      </c>
-      <c r="N51" t="s" s="2">
-        <v>486</v>
-      </c>
+        <v>491</v>
+      </c>
+      <c r="N51" s="2"/>
       <c r="O51" s="2"/>
       <c r="P51" t="s" s="2">
         <v>83</v>
@@ -8264,13 +8303,13 @@
         <v>83</v>
       </c>
       <c r="AF51" t="s" s="2">
-        <v>482</v>
+        <v>489</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH51" t="s" s="2">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="AI51" t="s" s="2">
         <v>83</v>
@@ -8288,10 +8327,10 @@
         <v>83</v>
       </c>
       <c r="AN51" t="s" s="2">
-        <v>487</v>
+        <v>461</v>
       </c>
       <c r="AO51" t="s" s="2">
-        <v>488</v>
+        <v>492</v>
       </c>
       <c r="AP51" t="s" s="2">
         <v>83</v>
@@ -8302,10 +8341,10 @@
     </row>
     <row r="52">
       <c r="A52" t="s" s="2">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
@@ -8328,16 +8367,16 @@
         <v>96</v>
       </c>
       <c r="K52" t="s" s="2">
-        <v>490</v>
+        <v>494</v>
       </c>
       <c r="L52" t="s" s="2">
-        <v>491</v>
+        <v>495</v>
       </c>
       <c r="M52" t="s" s="2">
-        <v>492</v>
+        <v>496</v>
       </c>
       <c r="N52" t="s" s="2">
-        <v>493</v>
+        <v>497</v>
       </c>
       <c r="O52" s="2"/>
       <c r="P52" t="s" s="2">
@@ -8387,7 +8426,7 @@
         <v>83</v>
       </c>
       <c r="AF52" t="s" s="2">
-        <v>489</v>
+        <v>493</v>
       </c>
       <c r="AG52" t="s" s="2">
         <v>81</v>
@@ -8411,10 +8450,10 @@
         <v>83</v>
       </c>
       <c r="AN52" t="s" s="2">
-        <v>487</v>
+        <v>498</v>
       </c>
       <c r="AO52" t="s" s="2">
-        <v>494</v>
+        <v>499</v>
       </c>
       <c r="AP52" t="s" s="2">
         <v>83</v>
@@ -8425,10 +8464,10 @@
     </row>
     <row r="53">
       <c r="A53" t="s" s="2">
-        <v>495</v>
+        <v>500</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>495</v>
+        <v>500</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -8451,20 +8490,18 @@
         <v>96</v>
       </c>
       <c r="K53" t="s" s="2">
-        <v>430</v>
+        <v>501</v>
       </c>
       <c r="L53" t="s" s="2">
-        <v>496</v>
+        <v>502</v>
       </c>
       <c r="M53" t="s" s="2">
-        <v>497</v>
+        <v>503</v>
       </c>
       <c r="N53" t="s" s="2">
-        <v>498</v>
-      </c>
-      <c r="O53" t="s" s="2">
-        <v>499</v>
-      </c>
+        <v>504</v>
+      </c>
+      <c r="O53" s="2"/>
       <c r="P53" t="s" s="2">
         <v>83</v>
       </c>
@@ -8512,7 +8549,7 @@
         <v>83</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>495</v>
+        <v>500</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>81</v>
@@ -8536,10 +8573,10 @@
         <v>83</v>
       </c>
       <c r="AN53" t="s" s="2">
-        <v>500</v>
+        <v>498</v>
       </c>
       <c r="AO53" t="s" s="2">
-        <v>501</v>
+        <v>505</v>
       </c>
       <c r="AP53" t="s" s="2">
         <v>83</v>
@@ -8550,10 +8587,10 @@
     </row>
     <row r="54">
       <c r="A54" t="s" s="2">
-        <v>502</v>
+        <v>506</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>502</v>
+        <v>506</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
@@ -8564,7 +8601,7 @@
         <v>81</v>
       </c>
       <c r="G54" t="s" s="2">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="H54" t="s" s="2">
         <v>83</v>
@@ -8573,19 +8610,23 @@
         <v>83</v>
       </c>
       <c r="J54" t="s" s="2">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="K54" t="s" s="2">
-        <v>172</v>
+        <v>441</v>
       </c>
       <c r="L54" t="s" s="2">
-        <v>173</v>
+        <v>507</v>
       </c>
       <c r="M54" t="s" s="2">
-        <v>174</v>
-      </c>
-      <c r="N54" s="2"/>
-      <c r="O54" s="2"/>
+        <v>508</v>
+      </c>
+      <c r="N54" t="s" s="2">
+        <v>509</v>
+      </c>
+      <c r="O54" t="s" s="2">
+        <v>510</v>
+      </c>
       <c r="P54" t="s" s="2">
         <v>83</v>
       </c>
@@ -8633,19 +8674,19 @@
         <v>83</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>175</v>
+        <v>506</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH54" t="s" s="2">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="AI54" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AJ54" t="s" s="2">
-        <v>83</v>
+        <v>107</v>
       </c>
       <c r="AK54" t="s" s="2">
         <v>83</v>
@@ -8657,10 +8698,10 @@
         <v>83</v>
       </c>
       <c r="AN54" t="s" s="2">
-        <v>83</v>
+        <v>511</v>
       </c>
       <c r="AO54" t="s" s="2">
-        <v>176</v>
+        <v>512</v>
       </c>
       <c r="AP54" t="s" s="2">
         <v>83</v>
@@ -8671,21 +8712,21 @@
     </row>
     <row r="55">
       <c r="A55" t="s" s="2">
-        <v>503</v>
+        <v>513</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>503</v>
+        <v>513</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
-        <v>155</v>
+        <v>83</v>
       </c>
       <c r="E55" s="2"/>
       <c r="F55" t="s" s="2">
         <v>81</v>
       </c>
       <c r="G55" t="s" s="2">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="H55" t="s" s="2">
         <v>83</v>
@@ -8697,17 +8738,15 @@
         <v>83</v>
       </c>
       <c r="K55" t="s" s="2">
-        <v>140</v>
+        <v>175</v>
       </c>
       <c r="L55" t="s" s="2">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="M55" t="s" s="2">
-        <v>179</v>
-      </c>
-      <c r="N55" t="s" s="2">
-        <v>158</v>
-      </c>
+        <v>177</v>
+      </c>
+      <c r="N55" s="2"/>
       <c r="O55" s="2"/>
       <c r="P55" t="s" s="2">
         <v>83</v>
@@ -8756,19 +8795,19 @@
         <v>83</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH55" t="s" s="2">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="AI55" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AJ55" t="s" s="2">
-        <v>146</v>
+        <v>83</v>
       </c>
       <c r="AK55" t="s" s="2">
         <v>83</v>
@@ -8783,7 +8822,7 @@
         <v>83</v>
       </c>
       <c r="AO55" t="s" s="2">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="AP55" t="s" s="2">
         <v>83</v>
@@ -8794,14 +8833,14 @@
     </row>
     <row r="56">
       <c r="A56" t="s" s="2">
-        <v>504</v>
+        <v>514</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>504</v>
+        <v>514</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" t="s" s="2">
-        <v>441</v>
+        <v>155</v>
       </c>
       <c r="E56" s="2"/>
       <c r="F56" t="s" s="2">
@@ -8814,26 +8853,24 @@
         <v>83</v>
       </c>
       <c r="I56" t="s" s="2">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="J56" t="s" s="2">
-        <v>96</v>
+        <v>83</v>
       </c>
       <c r="K56" t="s" s="2">
         <v>140</v>
       </c>
       <c r="L56" t="s" s="2">
-        <v>442</v>
+        <v>182</v>
       </c>
       <c r="M56" t="s" s="2">
-        <v>443</v>
+        <v>183</v>
       </c>
       <c r="N56" t="s" s="2">
         <v>158</v>
       </c>
-      <c r="O56" t="s" s="2">
-        <v>159</v>
-      </c>
+      <c r="O56" s="2"/>
       <c r="P56" t="s" s="2">
         <v>83</v>
       </c>
@@ -8881,7 +8918,7 @@
         <v>83</v>
       </c>
       <c r="AF56" t="s" s="2">
-        <v>444</v>
+        <v>185</v>
       </c>
       <c r="AG56" t="s" s="2">
         <v>81</v>
@@ -8908,7 +8945,7 @@
         <v>83</v>
       </c>
       <c r="AO56" t="s" s="2">
-        <v>138</v>
+        <v>179</v>
       </c>
       <c r="AP56" t="s" s="2">
         <v>83</v>
@@ -8919,45 +8956,45 @@
     </row>
     <row r="57">
       <c r="A57" t="s" s="2">
-        <v>505</v>
+        <v>515</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>505</v>
+        <v>515</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
-        <v>83</v>
+        <v>452</v>
       </c>
       <c r="E57" s="2"/>
       <c r="F57" t="s" s="2">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="G57" t="s" s="2">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="H57" t="s" s="2">
         <v>83</v>
       </c>
       <c r="I57" t="s" s="2">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="J57" t="s" s="2">
         <v>96</v>
       </c>
       <c r="K57" t="s" s="2">
-        <v>193</v>
+        <v>140</v>
       </c>
       <c r="L57" t="s" s="2">
-        <v>506</v>
+        <v>453</v>
       </c>
       <c r="M57" t="s" s="2">
-        <v>507</v>
+        <v>454</v>
       </c>
       <c r="N57" t="s" s="2">
-        <v>508</v>
+        <v>158</v>
       </c>
       <c r="O57" t="s" s="2">
-        <v>280</v>
+        <v>159</v>
       </c>
       <c r="P57" t="s" s="2">
         <v>83</v>
@@ -8982,13 +9019,13 @@
         <v>83</v>
       </c>
       <c r="X57" t="s" s="2">
-        <v>282</v>
+        <v>83</v>
       </c>
       <c r="Y57" t="s" s="2">
-        <v>283</v>
+        <v>83</v>
       </c>
       <c r="Z57" t="s" s="2">
-        <v>284</v>
+        <v>83</v>
       </c>
       <c r="AA57" t="s" s="2">
         <v>83</v>
@@ -9006,19 +9043,19 @@
         <v>83</v>
       </c>
       <c r="AF57" t="s" s="2">
-        <v>505</v>
+        <v>455</v>
       </c>
       <c r="AG57" t="s" s="2">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="AH57" t="s" s="2">
-        <v>95</v>
+        <v>82</v>
       </c>
       <c r="AI57" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AJ57" t="s" s="2">
-        <v>107</v>
+        <v>146</v>
       </c>
       <c r="AK57" t="s" s="2">
         <v>83</v>
@@ -9027,16 +9064,16 @@
         <v>83</v>
       </c>
       <c r="AM57" t="s" s="2">
-        <v>509</v>
+        <v>83</v>
       </c>
       <c r="AN57" t="s" s="2">
-        <v>287</v>
+        <v>83</v>
       </c>
       <c r="AO57" t="s" s="2">
-        <v>288</v>
+        <v>138</v>
       </c>
       <c r="AP57" t="s" s="2">
-        <v>289</v>
+        <v>83</v>
       </c>
       <c r="AQ57" t="s" s="2">
         <v>83</v>
@@ -9044,10 +9081,10 @@
     </row>
     <row r="58">
       <c r="A58" t="s" s="2">
-        <v>510</v>
+        <v>516</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>510</v>
+        <v>516</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
@@ -9055,7 +9092,7 @@
       </c>
       <c r="E58" s="2"/>
       <c r="F58" t="s" s="2">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="G58" t="s" s="2">
         <v>95</v>
@@ -9070,19 +9107,19 @@
         <v>96</v>
       </c>
       <c r="K58" t="s" s="2">
-        <v>353</v>
+        <v>199</v>
       </c>
       <c r="L58" t="s" s="2">
-        <v>511</v>
+        <v>517</v>
       </c>
       <c r="M58" t="s" s="2">
-        <v>355</v>
+        <v>518</v>
       </c>
       <c r="N58" t="s" s="2">
-        <v>512</v>
+        <v>519</v>
       </c>
       <c r="O58" t="s" s="2">
-        <v>357</v>
+        <v>291</v>
       </c>
       <c r="P58" t="s" s="2">
         <v>83</v>
@@ -9107,13 +9144,13 @@
         <v>83</v>
       </c>
       <c r="X58" t="s" s="2">
-        <v>83</v>
+        <v>293</v>
       </c>
       <c r="Y58" t="s" s="2">
-        <v>83</v>
+        <v>294</v>
       </c>
       <c r="Z58" t="s" s="2">
-        <v>83</v>
+        <v>295</v>
       </c>
       <c r="AA58" t="s" s="2">
         <v>83</v>
@@ -9131,10 +9168,10 @@
         <v>83</v>
       </c>
       <c r="AF58" t="s" s="2">
-        <v>510</v>
+        <v>516</v>
       </c>
       <c r="AG58" t="s" s="2">
-        <v>81</v>
+        <v>95</v>
       </c>
       <c r="AH58" t="s" s="2">
         <v>95</v>
@@ -9152,27 +9189,27 @@
         <v>83</v>
       </c>
       <c r="AM58" t="s" s="2">
-        <v>513</v>
+        <v>520</v>
       </c>
       <c r="AN58" t="s" s="2">
-        <v>360</v>
+        <v>298</v>
       </c>
       <c r="AO58" t="s" s="2">
-        <v>361</v>
+        <v>299</v>
       </c>
       <c r="AP58" t="s" s="2">
-        <v>83</v>
+        <v>300</v>
       </c>
       <c r="AQ58" t="s" s="2">
-        <v>362</v>
+        <v>83</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="s" s="2">
-        <v>514</v>
+        <v>521</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>514</v>
+        <v>521</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
@@ -9192,22 +9229,22 @@
         <v>83</v>
       </c>
       <c r="J59" t="s" s="2">
-        <v>83</v>
+        <v>96</v>
       </c>
       <c r="K59" t="s" s="2">
-        <v>193</v>
+        <v>364</v>
       </c>
       <c r="L59" t="s" s="2">
-        <v>515</v>
+        <v>522</v>
       </c>
       <c r="M59" t="s" s="2">
-        <v>516</v>
+        <v>366</v>
       </c>
       <c r="N59" t="s" s="2">
-        <v>517</v>
+        <v>523</v>
       </c>
       <c r="O59" t="s" s="2">
-        <v>367</v>
+        <v>368</v>
       </c>
       <c r="P59" t="s" s="2">
         <v>83</v>
@@ -9232,13 +9269,13 @@
         <v>83</v>
       </c>
       <c r="X59" t="s" s="2">
-        <v>198</v>
+        <v>83</v>
       </c>
       <c r="Y59" t="s" s="2">
-        <v>368</v>
+        <v>83</v>
       </c>
       <c r="Z59" t="s" s="2">
-        <v>369</v>
+        <v>83</v>
       </c>
       <c r="AA59" t="s" s="2">
         <v>83</v>
@@ -9256,7 +9293,7 @@
         <v>83</v>
       </c>
       <c r="AF59" t="s" s="2">
-        <v>514</v>
+        <v>521</v>
       </c>
       <c r="AG59" t="s" s="2">
         <v>81</v>
@@ -9265,7 +9302,7 @@
         <v>95</v>
       </c>
       <c r="AI59" t="s" s="2">
-        <v>370</v>
+        <v>83</v>
       </c>
       <c r="AJ59" t="s" s="2">
         <v>107</v>
@@ -9277,38 +9314,38 @@
         <v>83</v>
       </c>
       <c r="AM59" t="s" s="2">
-        <v>83</v>
+        <v>524</v>
       </c>
       <c r="AN59" t="s" s="2">
-        <v>138</v>
+        <v>371</v>
       </c>
       <c r="AO59" t="s" s="2">
-        <v>371</v>
+        <v>372</v>
       </c>
       <c r="AP59" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AQ59" t="s" s="2">
-        <v>83</v>
+        <v>373</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s" s="2">
-        <v>518</v>
+        <v>525</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>518</v>
+        <v>525</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
-        <v>373</v>
+        <v>83</v>
       </c>
       <c r="E60" s="2"/>
       <c r="F60" t="s" s="2">
         <v>81</v>
       </c>
       <c r="G60" t="s" s="2">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="H60" t="s" s="2">
         <v>83</v>
@@ -9320,19 +9357,19 @@
         <v>83</v>
       </c>
       <c r="K60" t="s" s="2">
-        <v>193</v>
+        <v>199</v>
       </c>
       <c r="L60" t="s" s="2">
-        <v>374</v>
+        <v>526</v>
       </c>
       <c r="M60" t="s" s="2">
-        <v>375</v>
+        <v>527</v>
       </c>
       <c r="N60" t="s" s="2">
-        <v>376</v>
+        <v>528</v>
       </c>
       <c r="O60" t="s" s="2">
-        <v>377</v>
+        <v>378</v>
       </c>
       <c r="P60" t="s" s="2">
         <v>83</v>
@@ -9357,13 +9394,13 @@
         <v>83</v>
       </c>
       <c r="X60" t="s" s="2">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="Y60" t="s" s="2">
-        <v>378</v>
+        <v>379</v>
       </c>
       <c r="Z60" t="s" s="2">
-        <v>379</v>
+        <v>380</v>
       </c>
       <c r="AA60" t="s" s="2">
         <v>83</v>
@@ -9381,16 +9418,16 @@
         <v>83</v>
       </c>
       <c r="AF60" t="s" s="2">
-        <v>518</v>
+        <v>525</v>
       </c>
       <c r="AG60" t="s" s="2">
         <v>81</v>
       </c>
       <c r="AH60" t="s" s="2">
-        <v>82</v>
+        <v>95</v>
       </c>
       <c r="AI60" t="s" s="2">
-        <v>83</v>
+        <v>381</v>
       </c>
       <c r="AJ60" t="s" s="2">
         <v>107</v>
@@ -9402,10 +9439,10 @@
         <v>83</v>
       </c>
       <c r="AM60" t="s" s="2">
-        <v>380</v>
+        <v>83</v>
       </c>
       <c r="AN60" t="s" s="2">
-        <v>381</v>
+        <v>138</v>
       </c>
       <c r="AO60" t="s" s="2">
         <v>382</v>
@@ -9414,19 +9451,19 @@
         <v>83</v>
       </c>
       <c r="AQ60" t="s" s="2">
-        <v>383</v>
+        <v>83</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="s" s="2">
-        <v>519</v>
+        <v>529</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>519</v>
+        <v>529</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
-        <v>83</v>
+        <v>384</v>
       </c>
       <c r="E61" s="2"/>
       <c r="F61" t="s" s="2">
@@ -9445,19 +9482,19 @@
         <v>83</v>
       </c>
       <c r="K61" t="s" s="2">
-        <v>84</v>
+        <v>199</v>
       </c>
       <c r="L61" t="s" s="2">
-        <v>520</v>
+        <v>385</v>
       </c>
       <c r="M61" t="s" s="2">
-        <v>521</v>
+        <v>386</v>
       </c>
       <c r="N61" t="s" s="2">
-        <v>433</v>
+        <v>387</v>
       </c>
       <c r="O61" t="s" s="2">
-        <v>434</v>
+        <v>388</v>
       </c>
       <c r="P61" t="s" s="2">
         <v>83</v>
@@ -9482,13 +9519,13 @@
         <v>83</v>
       </c>
       <c r="X61" t="s" s="2">
-        <v>83</v>
+        <v>205</v>
       </c>
       <c r="Y61" t="s" s="2">
-        <v>83</v>
+        <v>389</v>
       </c>
       <c r="Z61" t="s" s="2">
-        <v>83</v>
+        <v>390</v>
       </c>
       <c r="AA61" t="s" s="2">
         <v>83</v>
@@ -9506,7 +9543,7 @@
         <v>83</v>
       </c>
       <c r="AF61" t="s" s="2">
-        <v>519</v>
+        <v>529</v>
       </c>
       <c r="AG61" t="s" s="2">
         <v>81</v>
@@ -9527,18 +9564,143 @@
         <v>83</v>
       </c>
       <c r="AM61" t="s" s="2">
-        <v>83</v>
+        <v>391</v>
       </c>
       <c r="AN61" t="s" s="2">
-        <v>436</v>
+        <v>392</v>
       </c>
       <c r="AO61" t="s" s="2">
-        <v>437</v>
+        <v>393</v>
       </c>
       <c r="AP61" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AQ61" t="s" s="2">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="s" s="2">
+        <v>530</v>
+      </c>
+      <c r="B62" t="s" s="2">
+        <v>530</v>
+      </c>
+      <c r="C62" s="2"/>
+      <c r="D62" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="E62" s="2"/>
+      <c r="F62" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="G62" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="H62" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="I62" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="J62" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="K62" t="s" s="2">
+        <v>84</v>
+      </c>
+      <c r="L62" t="s" s="2">
+        <v>531</v>
+      </c>
+      <c r="M62" t="s" s="2">
+        <v>532</v>
+      </c>
+      <c r="N62" t="s" s="2">
+        <v>444</v>
+      </c>
+      <c r="O62" t="s" s="2">
+        <v>445</v>
+      </c>
+      <c r="P62" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="Q62" s="2"/>
+      <c r="R62" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="S62" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="T62" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="U62" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="V62" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="W62" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="X62" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="Y62" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="Z62" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AA62" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AB62" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AC62" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AD62" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AE62" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AF62" t="s" s="2">
+        <v>530</v>
+      </c>
+      <c r="AG62" t="s" s="2">
+        <v>81</v>
+      </c>
+      <c r="AH62" t="s" s="2">
+        <v>82</v>
+      </c>
+      <c r="AI62" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AJ62" t="s" s="2">
+        <v>107</v>
+      </c>
+      <c r="AK62" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AL62" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AM62" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AN62" t="s" s="2">
+        <v>447</v>
+      </c>
+      <c r="AO62" t="s" s="2">
+        <v>448</v>
+      </c>
+      <c r="AP62" t="s" s="2">
+        <v>83</v>
+      </c>
+      <c r="AQ62" t="s" s="2">
         <v>83</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Ajout règle de gestion e1d68365b1401be4f96591634e9bec8644e9fda4
</commit_message>
<xml_diff>
--- a/449-contenu-fhir---ajout-des-objets-presenceabsence-et-repas/ig/StructureDefinition-tddui-observation-repas.xlsx
+++ b/449-contenu-fhir---ajout-des-objets-presenceabsence-et-repas/ig/StructureDefinition-tddui-observation-repas.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2475" uniqueCount="533">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2475" uniqueCount="535">
   <si>
     <t>Property</t>
   </si>
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-06-09T13:44:39+00:00</t>
+    <t>2026-06-11T13:38:26+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -555,6 +555,13 @@
   </si>
   <si>
     <t>Observation.identifier:idRepas</t>
+  </si>
+  <si>
+    <t>Identifiant du repas</t>
+  </si>
+  <si>
+    <t>ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
+ObservationRepasIdentifierFormat:l'identifiant du repas doit respecter le format : 3+FINESS/identifiantLocalUsagerESSMS-REPAS-numRepas {value.matches('^3[0-9]{9}/[A-Za-z0-9]+-REPAS-[A-Za-z0-9]+$')}</t>
   </si>
   <si>
     <t>Observation.identifier:idRepas.id</t>
@@ -3549,7 +3556,7 @@
         <v>162</v>
       </c>
       <c r="L13" t="s" s="2">
-        <v>163</v>
+        <v>173</v>
       </c>
       <c r="M13" t="s" s="2">
         <v>164</v>
@@ -3617,7 +3624,7 @@
         <v>83</v>
       </c>
       <c r="AJ13" t="s" s="2">
-        <v>107</v>
+        <v>174</v>
       </c>
       <c r="AK13" t="s" s="2">
         <v>83</v>
@@ -3643,10 +3650,10 @@
     </row>
     <row r="14">
       <c r="A14" t="s" s="2">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" t="s" s="2">
@@ -3669,13 +3676,13 @@
         <v>83</v>
       </c>
       <c r="K14" t="s" s="2">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="L14" t="s" s="2">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="M14" t="s" s="2">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
@@ -3726,7 +3733,7 @@
         <v>83</v>
       </c>
       <c r="AF14" t="s" s="2">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="AG14" t="s" s="2">
         <v>81</v>
@@ -3753,7 +3760,7 @@
         <v>83</v>
       </c>
       <c r="AO14" t="s" s="2">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="AP14" t="s" s="2">
         <v>83</v>
@@ -3764,10 +3771,10 @@
     </row>
     <row r="15">
       <c r="A15" t="s" s="2">
-        <v>180</v>
+        <v>182</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" t="s" s="2">
@@ -3793,10 +3800,10 @@
         <v>140</v>
       </c>
       <c r="L15" t="s" s="2">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="M15" t="s" s="2">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="N15" t="s" s="2">
         <v>158</v>
@@ -3840,7 +3847,7 @@
         <v>143</v>
       </c>
       <c r="AC15" t="s" s="2">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="AD15" t="s" s="2">
         <v>83</v>
@@ -3849,7 +3856,7 @@
         <v>144</v>
       </c>
       <c r="AF15" t="s" s="2">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="AG15" t="s" s="2">
         <v>81</v>
@@ -3876,7 +3883,7 @@
         <v>83</v>
       </c>
       <c r="AO15" t="s" s="2">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="AP15" t="s" s="2">
         <v>83</v>
@@ -3887,10 +3894,10 @@
     </row>
     <row r="16">
       <c r="A16" t="s" s="2">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" t="s" s="2">
@@ -3916,16 +3923,16 @@
         <v>115</v>
       </c>
       <c r="L16" t="s" s="2">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="M16" t="s" s="2">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="N16" t="s" s="2">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="O16" t="s" s="2">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="P16" t="s" s="2">
         <v>83</v>
@@ -3950,13 +3957,13 @@
         <v>83</v>
       </c>
       <c r="X16" t="s" s="2">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="Y16" t="s" s="2">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="Z16" t="s" s="2">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="AA16" t="s" s="2">
         <v>83</v>
@@ -3974,7 +3981,7 @@
         <v>83</v>
       </c>
       <c r="AF16" t="s" s="2">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="AG16" t="s" s="2">
         <v>81</v>
@@ -4001,7 +4008,7 @@
         <v>138</v>
       </c>
       <c r="AO16" t="s" s="2">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="AP16" t="s" s="2">
         <v>83</v>
@@ -4012,10 +4019,10 @@
     </row>
     <row r="17">
       <c r="A17" t="s" s="2">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -4038,19 +4045,19 @@
         <v>96</v>
       </c>
       <c r="K17" t="s" s="2">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="L17" t="s" s="2">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="M17" t="s" s="2">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="N17" t="s" s="2">
-        <v>202</v>
+        <v>204</v>
       </c>
       <c r="O17" t="s" s="2">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="P17" t="s" s="2">
         <v>83</v>
@@ -4060,7 +4067,7 @@
         <v>83</v>
       </c>
       <c r="S17" t="s" s="2">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="T17" t="s" s="2">
         <v>83</v>
@@ -4075,13 +4082,13 @@
         <v>83</v>
       </c>
       <c r="X17" t="s" s="2">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="Y17" t="s" s="2">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="Z17" t="s" s="2">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="AA17" t="s" s="2">
         <v>83</v>
@@ -4099,7 +4106,7 @@
         <v>83</v>
       </c>
       <c r="AF17" t="s" s="2">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="AG17" t="s" s="2">
         <v>81</v>
@@ -4123,10 +4130,10 @@
         <v>83</v>
       </c>
       <c r="AN17" t="s" s="2">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="AO17" t="s" s="2">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="AP17" t="s" s="2">
         <v>83</v>
@@ -4137,10 +4144,10 @@
     </row>
     <row r="18">
       <c r="A18" t="s" s="2">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
@@ -4166,16 +4173,16 @@
         <v>109</v>
       </c>
       <c r="L18" t="s" s="2">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="M18" t="s" s="2">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="N18" t="s" s="2">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="O18" t="s" s="2">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="P18" t="s" s="2">
         <v>83</v>
@@ -4185,10 +4192,10 @@
         <v>83</v>
       </c>
       <c r="S18" t="s" s="2">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="T18" t="s" s="2">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="U18" t="s" s="2">
         <v>83</v>
@@ -4224,7 +4231,7 @@
         <v>83</v>
       </c>
       <c r="AF18" t="s" s="2">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="AG18" t="s" s="2">
         <v>81</v>
@@ -4248,10 +4255,10 @@
         <v>83</v>
       </c>
       <c r="AN18" t="s" s="2">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="AO18" t="s" s="2">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="AP18" t="s" s="2">
         <v>83</v>
@@ -4262,10 +4269,10 @@
     </row>
     <row r="19">
       <c r="A19" t="s" s="2">
-        <v>221</v>
+        <v>223</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
@@ -4288,16 +4295,16 @@
         <v>96</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="N19" t="s" s="2">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="O19" s="2"/>
       <c r="P19" t="s" s="2">
@@ -4311,7 +4318,7 @@
         <v>83</v>
       </c>
       <c r="T19" t="s" s="2">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="U19" t="s" s="2">
         <v>83</v>
@@ -4347,7 +4354,7 @@
         <v>83</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>81</v>
@@ -4371,10 +4378,10 @@
         <v>83</v>
       </c>
       <c r="AN19" t="s" s="2">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="AO19" t="s" s="2">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="AP19" t="s" s="2">
         <v>83</v>
@@ -4385,10 +4392,10 @@
     </row>
     <row r="20">
       <c r="A20" t="s" s="2">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
@@ -4411,13 +4418,13 @@
         <v>96</v>
       </c>
       <c r="K20" t="s" s="2">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
@@ -4468,7 +4475,7 @@
         <v>83</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>81</v>
@@ -4492,10 +4499,10 @@
         <v>83</v>
       </c>
       <c r="AN20" t="s" s="2">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="AO20" t="s" s="2">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="AP20" t="s" s="2">
         <v>83</v>
@@ -4506,10 +4513,10 @@
     </row>
     <row r="21">
       <c r="A21" t="s" s="2">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" t="s" s="2">
@@ -4532,16 +4539,16 @@
         <v>96</v>
       </c>
       <c r="K21" t="s" s="2">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="N21" t="s" s="2">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="O21" s="2"/>
       <c r="P21" t="s" s="2">
@@ -4591,7 +4598,7 @@
         <v>83</v>
       </c>
       <c r="AF21" t="s" s="2">
-        <v>244</v>
+        <v>246</v>
       </c>
       <c r="AG21" t="s" s="2">
         <v>81</v>
@@ -4615,10 +4622,10 @@
         <v>83</v>
       </c>
       <c r="AN21" t="s" s="2">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="AO21" t="s" s="2">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="AP21" t="s" s="2">
         <v>83</v>
@@ -4629,14 +4636,14 @@
     </row>
     <row r="22">
       <c r="A22" t="s" s="2">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" t="s" s="2">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="E22" s="2"/>
       <c r="F22" t="s" s="2">
@@ -4655,17 +4662,17 @@
         <v>96</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="N22" s="2"/>
       <c r="O22" t="s" s="2">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="P22" t="s" s="2">
         <v>83</v>
@@ -4714,7 +4721,7 @@
         <v>83</v>
       </c>
       <c r="AF22" t="s" s="2">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="AG22" t="s" s="2">
         <v>81</v>
@@ -4732,16 +4739,16 @@
         <v>83</v>
       </c>
       <c r="AL22" t="s" s="2">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="AM22" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AN22" t="s" s="2">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="AO22" t="s" s="2">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="AP22" t="s" s="2">
         <v>83</v>
@@ -4752,14 +4759,14 @@
     </row>
     <row r="23">
       <c r="A23" t="s" s="2">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" t="s" s="2">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="E23" s="2"/>
       <c r="F23" t="s" s="2">
@@ -4778,16 +4785,16 @@
         <v>96</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="N23" t="s" s="2">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="O23" s="2"/>
       <c r="P23" t="s" s="2">
@@ -4837,7 +4844,7 @@
         <v>83</v>
       </c>
       <c r="AF23" t="s" s="2">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="AG23" t="s" s="2">
         <v>81</v>
@@ -4855,16 +4862,16 @@
         <v>83</v>
       </c>
       <c r="AL23" t="s" s="2">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="AM23" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AN23" t="s" s="2">
-        <v>263</v>
+        <v>265</v>
       </c>
       <c r="AO23" t="s" s="2">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="AP23" t="s" s="2">
         <v>83</v>
@@ -4875,10 +4882,10 @@
     </row>
     <row r="24">
       <c r="A24" t="s" s="2">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -4904,16 +4911,16 @@
         <v>115</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>267</v>
+        <v>269</v>
       </c>
       <c r="N24" t="s" s="2">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="O24" t="s" s="2">
-        <v>269</v>
+        <v>271</v>
       </c>
       <c r="P24" t="s" s="2">
         <v>83</v>
@@ -4938,13 +4945,13 @@
         <v>83</v>
       </c>
       <c r="X24" t="s" s="2">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="Y24" t="s" s="2">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="Z24" t="s" s="2">
-        <v>271</v>
+        <v>273</v>
       </c>
       <c r="AA24" t="s" s="2">
         <v>83</v>
@@ -4962,7 +4969,7 @@
         <v>83</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>95</v>
@@ -4980,19 +4987,19 @@
         <v>83</v>
       </c>
       <c r="AL24" t="s" s="2">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="AM24" t="s" s="2">
-        <v>273</v>
+        <v>275</v>
       </c>
       <c r="AN24" t="s" s="2">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="AO24" t="s" s="2">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="AP24" t="s" s="2">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="AQ24" t="s" s="2">
         <v>83</v>
@@ -5000,10 +5007,10 @@
     </row>
     <row r="25">
       <c r="A25" t="s" s="2">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
@@ -5026,19 +5033,19 @@
         <v>83</v>
       </c>
       <c r="K25" t="s" s="2">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="N25" t="s" s="2">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="O25" t="s" s="2">
-        <v>281</v>
+        <v>283</v>
       </c>
       <c r="P25" t="s" s="2">
         <v>83</v>
@@ -5063,11 +5070,11 @@
         <v>83</v>
       </c>
       <c r="X25" t="s" s="2">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="Y25" s="2"/>
       <c r="Z25" t="s" s="2">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="AA25" t="s" s="2">
         <v>83</v>
@@ -5085,7 +5092,7 @@
         <v>83</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>81</v>
@@ -5100,7 +5107,7 @@
         <v>107</v>
       </c>
       <c r="AK25" t="s" s="2">
-        <v>283</v>
+        <v>285</v>
       </c>
       <c r="AL25" t="s" s="2">
         <v>83</v>
@@ -5112,10 +5119,10 @@
         <v>83</v>
       </c>
       <c r="AO25" t="s" s="2">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="AP25" t="s" s="2">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="AQ25" t="s" s="2">
         <v>83</v>
@@ -5123,14 +5130,14 @@
     </row>
     <row r="26">
       <c r="A26" t="s" s="2">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
-        <v>287</v>
+        <v>289</v>
       </c>
       <c r="E26" s="2"/>
       <c r="F26" t="s" s="2">
@@ -5149,19 +5156,19 @@
         <v>96</v>
       </c>
       <c r="K26" t="s" s="2">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>288</v>
+        <v>290</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="N26" t="s" s="2">
-        <v>290</v>
+        <v>292</v>
       </c>
       <c r="O26" t="s" s="2">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="P26" t="s" s="2">
         <v>83</v>
@@ -5171,7 +5178,7 @@
         <v>83</v>
       </c>
       <c r="S26" t="s" s="2">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="T26" t="s" s="2">
         <v>83</v>
@@ -5186,13 +5193,13 @@
         <v>83</v>
       </c>
       <c r="X26" t="s" s="2">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="Y26" t="s" s="2">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="Z26" t="s" s="2">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="AA26" t="s" s="2">
         <v>83</v>
@@ -5210,7 +5217,7 @@
         <v>83</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>95</v>
@@ -5228,30 +5235,30 @@
         <v>83</v>
       </c>
       <c r="AL26" t="s" s="2">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="AM26" t="s" s="2">
-        <v>297</v>
+        <v>299</v>
       </c>
       <c r="AN26" t="s" s="2">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="AO26" t="s" s="2">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="AP26" t="s" s="2">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="AQ26" t="s" s="2">
-        <v>301</v>
+        <v>303</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="s" s="2">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
@@ -5274,19 +5281,19 @@
         <v>96</v>
       </c>
       <c r="K27" t="s" s="2">
-        <v>303</v>
+        <v>305</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>304</v>
+        <v>306</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>305</v>
+        <v>307</v>
       </c>
       <c r="N27" t="s" s="2">
-        <v>306</v>
+        <v>308</v>
       </c>
       <c r="O27" t="s" s="2">
-        <v>307</v>
+        <v>309</v>
       </c>
       <c r="P27" t="s" s="2">
         <v>83</v>
@@ -5335,7 +5342,7 @@
         <v>83</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>302</v>
+        <v>304</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>81</v>
@@ -5350,22 +5357,22 @@
         <v>107</v>
       </c>
       <c r="AK27" t="s" s="2">
-        <v>308</v>
+        <v>310</v>
       </c>
       <c r="AL27" t="s" s="2">
-        <v>309</v>
+        <v>311</v>
       </c>
       <c r="AM27" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AN27" t="s" s="2">
-        <v>310</v>
+        <v>312</v>
       </c>
       <c r="AO27" t="s" s="2">
-        <v>311</v>
+        <v>313</v>
       </c>
       <c r="AP27" t="s" s="2">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="AQ27" t="s" s="2">
         <v>83</v>
@@ -5373,10 +5380,10 @@
     </row>
     <row r="28">
       <c r="A28" t="s" s="2">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
@@ -5399,16 +5406,16 @@
         <v>96</v>
       </c>
       <c r="K28" t="s" s="2">
-        <v>314</v>
+        <v>316</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>315</v>
+        <v>317</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="N28" t="s" s="2">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="O28" s="2"/>
       <c r="P28" t="s" s="2">
@@ -5458,7 +5465,7 @@
         <v>83</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>81</v>
@@ -5482,13 +5489,13 @@
         <v>83</v>
       </c>
       <c r="AN28" t="s" s="2">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="AO28" t="s" s="2">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="AP28" t="s" s="2">
-        <v>312</v>
+        <v>314</v>
       </c>
       <c r="AQ28" t="s" s="2">
         <v>83</v>
@@ -5496,14 +5503,14 @@
     </row>
     <row r="29">
       <c r="A29" t="s" s="2">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
-        <v>320</v>
+        <v>322</v>
       </c>
       <c r="E29" s="2"/>
       <c r="F29" t="s" s="2">
@@ -5522,19 +5529,19 @@
         <v>96</v>
       </c>
       <c r="K29" t="s" s="2">
-        <v>321</v>
+        <v>323</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>322</v>
+        <v>324</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>323</v>
+        <v>325</v>
       </c>
       <c r="N29" t="s" s="2">
-        <v>324</v>
+        <v>326</v>
       </c>
       <c r="O29" t="s" s="2">
-        <v>325</v>
+        <v>327</v>
       </c>
       <c r="P29" t="s" s="2">
         <v>83</v>
@@ -5583,7 +5590,7 @@
         <v>83</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>81</v>
@@ -5601,19 +5608,19 @@
         <v>83</v>
       </c>
       <c r="AL29" t="s" s="2">
-        <v>326</v>
+        <v>328</v>
       </c>
       <c r="AM29" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AN29" t="s" s="2">
-        <v>327</v>
+        <v>329</v>
       </c>
       <c r="AO29" t="s" s="2">
-        <v>328</v>
+        <v>330</v>
       </c>
       <c r="AP29" t="s" s="2">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="AQ29" t="s" s="2">
         <v>83</v>
@@ -5621,14 +5628,14 @@
     </row>
     <row r="30">
       <c r="A30" t="s" s="2">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="E30" s="2"/>
       <c r="F30" t="s" s="2">
@@ -5647,19 +5654,19 @@
         <v>96</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="N30" t="s" s="2">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="O30" t="s" s="2">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="P30" t="s" s="2">
         <v>83</v>
@@ -5696,17 +5703,17 @@
         <v>83</v>
       </c>
       <c r="AB30" t="s" s="2">
-        <v>337</v>
+        <v>339</v>
       </c>
       <c r="AC30" s="2"/>
       <c r="AD30" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AE30" t="s" s="2">
-        <v>338</v>
+        <v>340</v>
       </c>
       <c r="AF30" t="s" s="2">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>81</v>
@@ -5724,19 +5731,19 @@
         <v>83</v>
       </c>
       <c r="AL30" t="s" s="2">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="AM30" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AN30" t="s" s="2">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="AO30" t="s" s="2">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="AP30" t="s" s="2">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="AQ30" t="s" s="2">
         <v>83</v>
@@ -5744,16 +5751,16 @@
     </row>
     <row r="31">
       <c r="A31" t="s" s="2">
-        <v>343</v>
+        <v>345</v>
       </c>
       <c r="B31" t="s" s="2">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="C31" t="s" s="2">
-        <v>344</v>
+        <v>346</v>
       </c>
       <c r="D31" t="s" s="2">
-        <v>331</v>
+        <v>333</v>
       </c>
       <c r="E31" s="2"/>
       <c r="F31" t="s" s="2">
@@ -5772,19 +5779,19 @@
         <v>96</v>
       </c>
       <c r="K31" t="s" s="2">
-        <v>332</v>
+        <v>334</v>
       </c>
       <c r="L31" t="s" s="2">
-        <v>333</v>
+        <v>335</v>
       </c>
       <c r="M31" t="s" s="2">
-        <v>334</v>
+        <v>336</v>
       </c>
       <c r="N31" t="s" s="2">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="O31" t="s" s="2">
-        <v>336</v>
+        <v>338</v>
       </c>
       <c r="P31" t="s" s="2">
         <v>83</v>
@@ -5833,7 +5840,7 @@
         <v>83</v>
       </c>
       <c r="AF31" t="s" s="2">
-        <v>330</v>
+        <v>332</v>
       </c>
       <c r="AG31" t="s" s="2">
         <v>81</v>
@@ -5848,22 +5855,22 @@
         <v>107</v>
       </c>
       <c r="AK31" t="s" s="2">
-        <v>345</v>
+        <v>347</v>
       </c>
       <c r="AL31" t="s" s="2">
-        <v>339</v>
+        <v>341</v>
       </c>
       <c r="AM31" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AN31" t="s" s="2">
-        <v>340</v>
+        <v>342</v>
       </c>
       <c r="AO31" t="s" s="2">
-        <v>341</v>
+        <v>343</v>
       </c>
       <c r="AP31" t="s" s="2">
-        <v>342</v>
+        <v>344</v>
       </c>
       <c r="AQ31" t="s" s="2">
         <v>83</v>
@@ -5871,10 +5878,10 @@
     </row>
     <row r="32">
       <c r="A32" t="s" s="2">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="B32" t="s" s="2">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" t="s" s="2">
@@ -5897,16 +5904,16 @@
         <v>96</v>
       </c>
       <c r="K32" t="s" s="2">
-        <v>347</v>
+        <v>349</v>
       </c>
       <c r="L32" t="s" s="2">
-        <v>348</v>
+        <v>350</v>
       </c>
       <c r="M32" t="s" s="2">
-        <v>349</v>
+        <v>351</v>
       </c>
       <c r="N32" t="s" s="2">
-        <v>350</v>
+        <v>352</v>
       </c>
       <c r="O32" s="2"/>
       <c r="P32" t="s" s="2">
@@ -5956,7 +5963,7 @@
         <v>83</v>
       </c>
       <c r="AF32" t="s" s="2">
-        <v>346</v>
+        <v>348</v>
       </c>
       <c r="AG32" t="s" s="2">
         <v>81</v>
@@ -5980,13 +5987,13 @@
         <v>83</v>
       </c>
       <c r="AN32" t="s" s="2">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="AO32" t="s" s="2">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="AP32" t="s" s="2">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="AQ32" t="s" s="2">
         <v>83</v>
@@ -5994,10 +6001,10 @@
     </row>
     <row r="33">
       <c r="A33" t="s" s="2">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="B33" t="s" s="2">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" t="s" s="2">
@@ -6020,17 +6027,17 @@
         <v>96</v>
       </c>
       <c r="K33" t="s" s="2">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="L33" t="s" s="2">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="M33" t="s" s="2">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="N33" s="2"/>
       <c r="O33" t="s" s="2">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="P33" t="s" s="2">
         <v>83</v>
@@ -6079,7 +6086,7 @@
         <v>83</v>
       </c>
       <c r="AF33" t="s" s="2">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="AG33" t="s" s="2">
         <v>81</v>
@@ -6097,19 +6104,19 @@
         <v>83</v>
       </c>
       <c r="AL33" t="s" s="2">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="AM33" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AN33" t="s" s="2">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="AO33" t="s" s="2">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="AP33" t="s" s="2">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="AQ33" t="s" s="2">
         <v>83</v>
@@ -6117,10 +6124,10 @@
     </row>
     <row r="34">
       <c r="A34" t="s" s="2">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="B34" t="s" s="2">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" t="s" s="2">
@@ -6143,19 +6150,19 @@
         <v>96</v>
       </c>
       <c r="K34" t="s" s="2">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="L34" t="s" s="2">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="M34" t="s" s="2">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="N34" t="s" s="2">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="O34" t="s" s="2">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="P34" t="s" s="2">
         <v>83</v>
@@ -6204,7 +6211,7 @@
         <v>83</v>
       </c>
       <c r="AF34" t="s" s="2">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="AG34" t="s" s="2">
         <v>81</v>
@@ -6213,7 +6220,7 @@
         <v>95</v>
       </c>
       <c r="AI34" t="s" s="2">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="AJ34" t="s" s="2">
         <v>107</v>
@@ -6225,27 +6232,27 @@
         <v>83</v>
       </c>
       <c r="AM34" t="s" s="2">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="AN34" t="s" s="2">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="AO34" t="s" s="2">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="AP34" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AQ34" t="s" s="2">
-        <v>373</v>
+        <v>375</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="s" s="2">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="B35" t="s" s="2">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" t="s" s="2">
@@ -6268,19 +6275,19 @@
         <v>83</v>
       </c>
       <c r="K35" t="s" s="2">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="L35" t="s" s="2">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="M35" t="s" s="2">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="N35" t="s" s="2">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="O35" t="s" s="2">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="P35" t="s" s="2">
         <v>83</v>
@@ -6305,13 +6312,13 @@
         <v>83</v>
       </c>
       <c r="X35" t="s" s="2">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="Y35" t="s" s="2">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="Z35" t="s" s="2">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="AA35" t="s" s="2">
         <v>83</v>
@@ -6329,7 +6336,7 @@
         <v>83</v>
       </c>
       <c r="AF35" t="s" s="2">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="AG35" t="s" s="2">
         <v>81</v>
@@ -6338,7 +6345,7 @@
         <v>95</v>
       </c>
       <c r="AI35" t="s" s="2">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="AJ35" t="s" s="2">
         <v>107</v>
@@ -6356,7 +6363,7 @@
         <v>138</v>
       </c>
       <c r="AO35" t="s" s="2">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="AP35" t="s" s="2">
         <v>83</v>
@@ -6367,14 +6374,14 @@
     </row>
     <row r="36">
       <c r="A36" t="s" s="2">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="B36" t="s" s="2">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" t="s" s="2">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="E36" s="2"/>
       <c r="F36" t="s" s="2">
@@ -6393,19 +6400,19 @@
         <v>83</v>
       </c>
       <c r="K36" t="s" s="2">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="L36" t="s" s="2">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="M36" t="s" s="2">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="N36" t="s" s="2">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="O36" t="s" s="2">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="P36" t="s" s="2">
         <v>83</v>
@@ -6430,13 +6437,13 @@
         <v>83</v>
       </c>
       <c r="X36" t="s" s="2">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="Y36" t="s" s="2">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="Z36" t="s" s="2">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="AA36" t="s" s="2">
         <v>83</v>
@@ -6454,7 +6461,7 @@
         <v>83</v>
       </c>
       <c r="AF36" t="s" s="2">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="AG36" t="s" s="2">
         <v>81</v>
@@ -6475,27 +6482,27 @@
         <v>83</v>
       </c>
       <c r="AM36" t="s" s="2">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="AN36" t="s" s="2">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="AO36" t="s" s="2">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="AP36" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AQ36" t="s" s="2">
-        <v>394</v>
+        <v>396</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="s" s="2">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="B37" t="s" s="2">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" t="s" s="2">
@@ -6518,19 +6525,19 @@
         <v>83</v>
       </c>
       <c r="K37" t="s" s="2">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="L37" t="s" s="2">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="M37" t="s" s="2">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="N37" t="s" s="2">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="O37" t="s" s="2">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="P37" t="s" s="2">
         <v>83</v>
@@ -6579,7 +6586,7 @@
         <v>83</v>
       </c>
       <c r="AF37" t="s" s="2">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="AG37" t="s" s="2">
         <v>81</v>
@@ -6603,10 +6610,10 @@
         <v>83</v>
       </c>
       <c r="AN37" t="s" s="2">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="AO37" t="s" s="2">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="AP37" t="s" s="2">
         <v>83</v>
@@ -6617,10 +6624,10 @@
     </row>
     <row r="38">
       <c r="A38" t="s" s="2">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="B38" t="s" s="2">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="C38" s="2"/>
       <c r="D38" t="s" s="2">
@@ -6643,16 +6650,16 @@
         <v>83</v>
       </c>
       <c r="K38" t="s" s="2">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="L38" t="s" s="2">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="M38" t="s" s="2">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="N38" t="s" s="2">
-        <v>406</v>
+        <v>408</v>
       </c>
       <c r="O38" s="2"/>
       <c r="P38" t="s" s="2">
@@ -6678,13 +6685,13 @@
         <v>83</v>
       </c>
       <c r="X38" t="s" s="2">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="Y38" t="s" s="2">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="Z38" t="s" s="2">
-        <v>408</v>
+        <v>410</v>
       </c>
       <c r="AA38" t="s" s="2">
         <v>83</v>
@@ -6702,7 +6709,7 @@
         <v>83</v>
       </c>
       <c r="AF38" t="s" s="2">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="AG38" t="s" s="2">
         <v>81</v>
@@ -6723,27 +6730,27 @@
         <v>83</v>
       </c>
       <c r="AM38" t="s" s="2">
-        <v>409</v>
+        <v>411</v>
       </c>
       <c r="AN38" t="s" s="2">
-        <v>410</v>
+        <v>412</v>
       </c>
       <c r="AO38" t="s" s="2">
-        <v>411</v>
+        <v>413</v>
       </c>
       <c r="AP38" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AQ38" t="s" s="2">
-        <v>412</v>
+        <v>414</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s" s="2">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="B39" t="s" s="2">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="C39" s="2"/>
       <c r="D39" t="s" s="2">
@@ -6766,19 +6773,19 @@
         <v>83</v>
       </c>
       <c r="K39" t="s" s="2">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="L39" t="s" s="2">
-        <v>414</v>
+        <v>416</v>
       </c>
       <c r="M39" t="s" s="2">
-        <v>415</v>
+        <v>417</v>
       </c>
       <c r="N39" t="s" s="2">
-        <v>416</v>
+        <v>418</v>
       </c>
       <c r="O39" t="s" s="2">
-        <v>417</v>
+        <v>419</v>
       </c>
       <c r="P39" t="s" s="2">
         <v>83</v>
@@ -6803,13 +6810,13 @@
         <v>83</v>
       </c>
       <c r="X39" t="s" s="2">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="Y39" t="s" s="2">
-        <v>418</v>
+        <v>420</v>
       </c>
       <c r="Z39" t="s" s="2">
-        <v>419</v>
+        <v>421</v>
       </c>
       <c r="AA39" t="s" s="2">
         <v>83</v>
@@ -6827,7 +6834,7 @@
         <v>83</v>
       </c>
       <c r="AF39" t="s" s="2">
-        <v>413</v>
+        <v>415</v>
       </c>
       <c r="AG39" t="s" s="2">
         <v>81</v>
@@ -6851,10 +6858,10 @@
         <v>83</v>
       </c>
       <c r="AN39" t="s" s="2">
-        <v>420</v>
+        <v>422</v>
       </c>
       <c r="AO39" t="s" s="2">
-        <v>421</v>
+        <v>423</v>
       </c>
       <c r="AP39" t="s" s="2">
         <v>83</v>
@@ -6865,10 +6872,10 @@
     </row>
     <row r="40">
       <c r="A40" t="s" s="2">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="B40" t="s" s="2">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" t="s" s="2">
@@ -6891,16 +6898,16 @@
         <v>83</v>
       </c>
       <c r="K40" t="s" s="2">
-        <v>423</v>
+        <v>425</v>
       </c>
       <c r="L40" t="s" s="2">
-        <v>424</v>
+        <v>426</v>
       </c>
       <c r="M40" t="s" s="2">
-        <v>425</v>
+        <v>427</v>
       </c>
       <c r="N40" t="s" s="2">
-        <v>426</v>
+        <v>428</v>
       </c>
       <c r="O40" s="2"/>
       <c r="P40" t="s" s="2">
@@ -6950,7 +6957,7 @@
         <v>83</v>
       </c>
       <c r="AF40" t="s" s="2">
-        <v>422</v>
+        <v>424</v>
       </c>
       <c r="AG40" t="s" s="2">
         <v>81</v>
@@ -6971,27 +6978,27 @@
         <v>83</v>
       </c>
       <c r="AM40" t="s" s="2">
-        <v>427</v>
+        <v>429</v>
       </c>
       <c r="AN40" t="s" s="2">
-        <v>428</v>
+        <v>430</v>
       </c>
       <c r="AO40" t="s" s="2">
-        <v>429</v>
+        <v>431</v>
       </c>
       <c r="AP40" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AQ40" t="s" s="2">
-        <v>430</v>
+        <v>432</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="s" s="2">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="B41" t="s" s="2">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" t="s" s="2">
@@ -7014,16 +7021,16 @@
         <v>83</v>
       </c>
       <c r="K41" t="s" s="2">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="L41" t="s" s="2">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="M41" t="s" s="2">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="N41" t="s" s="2">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="O41" s="2"/>
       <c r="P41" t="s" s="2">
@@ -7073,7 +7080,7 @@
         <v>83</v>
       </c>
       <c r="AF41" t="s" s="2">
-        <v>431</v>
+        <v>433</v>
       </c>
       <c r="AG41" t="s" s="2">
         <v>81</v>
@@ -7094,27 +7101,27 @@
         <v>83</v>
       </c>
       <c r="AM41" t="s" s="2">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="AN41" t="s" s="2">
-        <v>437</v>
+        <v>439</v>
       </c>
       <c r="AO41" t="s" s="2">
-        <v>438</v>
+        <v>440</v>
       </c>
       <c r="AP41" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AQ41" t="s" s="2">
-        <v>439</v>
+        <v>441</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="s" s="2">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="B42" t="s" s="2">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" t="s" s="2">
@@ -7137,19 +7144,19 @@
         <v>83</v>
       </c>
       <c r="K42" t="s" s="2">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="L42" t="s" s="2">
-        <v>442</v>
+        <v>444</v>
       </c>
       <c r="M42" t="s" s="2">
-        <v>443</v>
+        <v>445</v>
       </c>
       <c r="N42" t="s" s="2">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="O42" t="s" s="2">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="P42" t="s" s="2">
         <v>83</v>
@@ -7198,7 +7205,7 @@
         <v>83</v>
       </c>
       <c r="AF42" t="s" s="2">
-        <v>440</v>
+        <v>442</v>
       </c>
       <c r="AG42" t="s" s="2">
         <v>81</v>
@@ -7210,7 +7217,7 @@
         <v>83</v>
       </c>
       <c r="AJ42" t="s" s="2">
-        <v>446</v>
+        <v>448</v>
       </c>
       <c r="AK42" t="s" s="2">
         <v>83</v>
@@ -7222,10 +7229,10 @@
         <v>83</v>
       </c>
       <c r="AN42" t="s" s="2">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="AO42" t="s" s="2">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="AP42" t="s" s="2">
         <v>83</v>
@@ -7236,10 +7243,10 @@
     </row>
     <row r="43">
       <c r="A43" t="s" s="2">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="B43" t="s" s="2">
-        <v>449</v>
+        <v>451</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" t="s" s="2">
@@ -7262,13 +7269,13 @@
         <v>83</v>
       </c>
       <c r="K43" t="s" s="2">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="L43" t="s" s="2">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="M43" t="s" s="2">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="N43" s="2"/>
       <c r="O43" s="2"/>
@@ -7319,7 +7326,7 @@
         <v>83</v>
       </c>
       <c r="AF43" t="s" s="2">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="AG43" t="s" s="2">
         <v>81</v>
@@ -7346,7 +7353,7 @@
         <v>83</v>
       </c>
       <c r="AO43" t="s" s="2">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="AP43" t="s" s="2">
         <v>83</v>
@@ -7357,10 +7364,10 @@
     </row>
     <row r="44">
       <c r="A44" t="s" s="2">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="B44" t="s" s="2">
-        <v>450</v>
+        <v>452</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" t="s" s="2">
@@ -7386,10 +7393,10 @@
         <v>140</v>
       </c>
       <c r="L44" t="s" s="2">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="M44" t="s" s="2">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="N44" t="s" s="2">
         <v>158</v>
@@ -7442,7 +7449,7 @@
         <v>83</v>
       </c>
       <c r="AF44" t="s" s="2">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="AG44" t="s" s="2">
         <v>81</v>
@@ -7469,7 +7476,7 @@
         <v>83</v>
       </c>
       <c r="AO44" t="s" s="2">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="AP44" t="s" s="2">
         <v>83</v>
@@ -7480,14 +7487,14 @@
     </row>
     <row r="45">
       <c r="A45" t="s" s="2">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="B45" t="s" s="2">
-        <v>451</v>
+        <v>453</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" t="s" s="2">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="E45" s="2"/>
       <c r="F45" t="s" s="2">
@@ -7509,10 +7516,10 @@
         <v>140</v>
       </c>
       <c r="L45" t="s" s="2">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="M45" t="s" s="2">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="N45" t="s" s="2">
         <v>158</v>
@@ -7567,7 +7574,7 @@
         <v>83</v>
       </c>
       <c r="AF45" t="s" s="2">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="AG45" t="s" s="2">
         <v>81</v>
@@ -7605,10 +7612,10 @@
     </row>
     <row r="46">
       <c r="A46" t="s" s="2">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="B46" t="s" s="2">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" t="s" s="2">
@@ -7631,13 +7638,13 @@
         <v>83</v>
       </c>
       <c r="K46" t="s" s="2">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="L46" t="s" s="2">
-        <v>458</v>
+        <v>460</v>
       </c>
       <c r="M46" t="s" s="2">
-        <v>459</v>
+        <v>461</v>
       </c>
       <c r="N46" s="2"/>
       <c r="O46" s="2"/>
@@ -7688,7 +7695,7 @@
         <v>83</v>
       </c>
       <c r="AF46" t="s" s="2">
-        <v>456</v>
+        <v>458</v>
       </c>
       <c r="AG46" t="s" s="2">
         <v>81</v>
@@ -7697,7 +7704,7 @@
         <v>95</v>
       </c>
       <c r="AI46" t="s" s="2">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="AJ46" t="s" s="2">
         <v>107</v>
@@ -7712,10 +7719,10 @@
         <v>83</v>
       </c>
       <c r="AN46" t="s" s="2">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="AO46" t="s" s="2">
-        <v>462</v>
+        <v>464</v>
       </c>
       <c r="AP46" t="s" s="2">
         <v>83</v>
@@ -7726,10 +7733,10 @@
     </row>
     <row r="47">
       <c r="A47" t="s" s="2">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="B47" t="s" s="2">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="C47" s="2"/>
       <c r="D47" t="s" s="2">
@@ -7752,13 +7759,13 @@
         <v>83</v>
       </c>
       <c r="K47" t="s" s="2">
-        <v>457</v>
+        <v>459</v>
       </c>
       <c r="L47" t="s" s="2">
-        <v>464</v>
+        <v>466</v>
       </c>
       <c r="M47" t="s" s="2">
-        <v>465</v>
+        <v>467</v>
       </c>
       <c r="N47" s="2"/>
       <c r="O47" s="2"/>
@@ -7809,7 +7816,7 @@
         <v>83</v>
       </c>
       <c r="AF47" t="s" s="2">
-        <v>463</v>
+        <v>465</v>
       </c>
       <c r="AG47" t="s" s="2">
         <v>81</v>
@@ -7818,7 +7825,7 @@
         <v>95</v>
       </c>
       <c r="AI47" t="s" s="2">
-        <v>460</v>
+        <v>462</v>
       </c>
       <c r="AJ47" t="s" s="2">
         <v>107</v>
@@ -7833,10 +7840,10 @@
         <v>83</v>
       </c>
       <c r="AN47" t="s" s="2">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="AO47" t="s" s="2">
-        <v>466</v>
+        <v>468</v>
       </c>
       <c r="AP47" t="s" s="2">
         <v>83</v>
@@ -7847,10 +7854,10 @@
     </row>
     <row r="48">
       <c r="A48" t="s" s="2">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="B48" t="s" s="2">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" t="s" s="2">
@@ -7873,19 +7880,19 @@
         <v>83</v>
       </c>
       <c r="K48" t="s" s="2">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="L48" t="s" s="2">
-        <v>468</v>
+        <v>470</v>
       </c>
       <c r="M48" t="s" s="2">
-        <v>469</v>
+        <v>471</v>
       </c>
       <c r="N48" t="s" s="2">
-        <v>470</v>
+        <v>472</v>
       </c>
       <c r="O48" t="s" s="2">
-        <v>471</v>
+        <v>473</v>
       </c>
       <c r="P48" t="s" s="2">
         <v>83</v>
@@ -7913,10 +7920,10 @@
         <v>119</v>
       </c>
       <c r="Y48" t="s" s="2">
-        <v>472</v>
+        <v>474</v>
       </c>
       <c r="Z48" t="s" s="2">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="AA48" t="s" s="2">
         <v>83</v>
@@ -7934,7 +7941,7 @@
         <v>83</v>
       </c>
       <c r="AF48" t="s" s="2">
-        <v>467</v>
+        <v>469</v>
       </c>
       <c r="AG48" t="s" s="2">
         <v>81</v>
@@ -7955,13 +7962,13 @@
         <v>83</v>
       </c>
       <c r="AM48" t="s" s="2">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="AN48" t="s" s="2">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="AO48" t="s" s="2">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="AP48" t="s" s="2">
         <v>83</v>
@@ -7972,10 +7979,10 @@
     </row>
     <row r="49">
       <c r="A49" t="s" s="2">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="B49" t="s" s="2">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" t="s" s="2">
@@ -7998,19 +8005,19 @@
         <v>83</v>
       </c>
       <c r="K49" t="s" s="2">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="L49" t="s" s="2">
-        <v>477</v>
+        <v>479</v>
       </c>
       <c r="M49" t="s" s="2">
-        <v>478</v>
+        <v>480</v>
       </c>
       <c r="N49" t="s" s="2">
-        <v>479</v>
+        <v>481</v>
       </c>
       <c r="O49" t="s" s="2">
-        <v>480</v>
+        <v>482</v>
       </c>
       <c r="P49" t="s" s="2">
         <v>83</v>
@@ -8035,13 +8042,13 @@
         <v>83</v>
       </c>
       <c r="X49" t="s" s="2">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="Y49" t="s" s="2">
-        <v>481</v>
+        <v>483</v>
       </c>
       <c r="Z49" t="s" s="2">
-        <v>482</v>
+        <v>484</v>
       </c>
       <c r="AA49" t="s" s="2">
         <v>83</v>
@@ -8059,7 +8066,7 @@
         <v>83</v>
       </c>
       <c r="AF49" t="s" s="2">
-        <v>476</v>
+        <v>478</v>
       </c>
       <c r="AG49" t="s" s="2">
         <v>81</v>
@@ -8080,13 +8087,13 @@
         <v>83</v>
       </c>
       <c r="AM49" t="s" s="2">
-        <v>474</v>
+        <v>476</v>
       </c>
       <c r="AN49" t="s" s="2">
-        <v>475</v>
+        <v>477</v>
       </c>
       <c r="AO49" t="s" s="2">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="AP49" t="s" s="2">
         <v>83</v>
@@ -8097,10 +8104,10 @@
     </row>
     <row r="50">
       <c r="A50" t="s" s="2">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="B50" t="s" s="2">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" t="s" s="2">
@@ -8123,17 +8130,17 @@
         <v>83</v>
       </c>
       <c r="K50" t="s" s="2">
-        <v>484</v>
+        <v>486</v>
       </c>
       <c r="L50" t="s" s="2">
-        <v>485</v>
+        <v>487</v>
       </c>
       <c r="M50" t="s" s="2">
-        <v>486</v>
+        <v>488</v>
       </c>
       <c r="N50" s="2"/>
       <c r="O50" t="s" s="2">
-        <v>487</v>
+        <v>489</v>
       </c>
       <c r="P50" t="s" s="2">
         <v>83</v>
@@ -8182,7 +8189,7 @@
         <v>83</v>
       </c>
       <c r="AF50" t="s" s="2">
-        <v>483</v>
+        <v>485</v>
       </c>
       <c r="AG50" t="s" s="2">
         <v>81</v>
@@ -8209,7 +8216,7 @@
         <v>83</v>
       </c>
       <c r="AO50" t="s" s="2">
-        <v>488</v>
+        <v>490</v>
       </c>
       <c r="AP50" t="s" s="2">
         <v>83</v>
@@ -8220,10 +8227,10 @@
     </row>
     <row r="51">
       <c r="A51" t="s" s="2">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="B51" t="s" s="2">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" t="s" s="2">
@@ -8246,13 +8253,13 @@
         <v>83</v>
       </c>
       <c r="K51" t="s" s="2">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="L51" t="s" s="2">
-        <v>490</v>
+        <v>492</v>
       </c>
       <c r="M51" t="s" s="2">
-        <v>491</v>
+        <v>493</v>
       </c>
       <c r="N51" s="2"/>
       <c r="O51" s="2"/>
@@ -8303,7 +8310,7 @@
         <v>83</v>
       </c>
       <c r="AF51" t="s" s="2">
-        <v>489</v>
+        <v>491</v>
       </c>
       <c r="AG51" t="s" s="2">
         <v>81</v>
@@ -8327,10 +8334,10 @@
         <v>83</v>
       </c>
       <c r="AN51" t="s" s="2">
-        <v>461</v>
+        <v>463</v>
       </c>
       <c r="AO51" t="s" s="2">
-        <v>492</v>
+        <v>494</v>
       </c>
       <c r="AP51" t="s" s="2">
         <v>83</v>
@@ -8341,10 +8348,10 @@
     </row>
     <row r="52">
       <c r="A52" t="s" s="2">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="B52" t="s" s="2">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" t="s" s="2">
@@ -8367,16 +8374,16 @@
         <v>96</v>
       </c>
       <c r="K52" t="s" s="2">
-        <v>494</v>
+        <v>496</v>
       </c>
       <c r="L52" t="s" s="2">
-        <v>495</v>
+        <v>497</v>
       </c>
       <c r="M52" t="s" s="2">
-        <v>496</v>
+        <v>498</v>
       </c>
       <c r="N52" t="s" s="2">
-        <v>497</v>
+        <v>499</v>
       </c>
       <c r="O52" s="2"/>
       <c r="P52" t="s" s="2">
@@ -8426,7 +8433,7 @@
         <v>83</v>
       </c>
       <c r="AF52" t="s" s="2">
-        <v>493</v>
+        <v>495</v>
       </c>
       <c r="AG52" t="s" s="2">
         <v>81</v>
@@ -8450,10 +8457,10 @@
         <v>83</v>
       </c>
       <c r="AN52" t="s" s="2">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="AO52" t="s" s="2">
-        <v>499</v>
+        <v>501</v>
       </c>
       <c r="AP52" t="s" s="2">
         <v>83</v>
@@ -8464,10 +8471,10 @@
     </row>
     <row r="53">
       <c r="A53" t="s" s="2">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="B53" t="s" s="2">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" t="s" s="2">
@@ -8490,16 +8497,16 @@
         <v>96</v>
       </c>
       <c r="K53" t="s" s="2">
-        <v>501</v>
+        <v>503</v>
       </c>
       <c r="L53" t="s" s="2">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="M53" t="s" s="2">
-        <v>503</v>
+        <v>505</v>
       </c>
       <c r="N53" t="s" s="2">
-        <v>504</v>
+        <v>506</v>
       </c>
       <c r="O53" s="2"/>
       <c r="P53" t="s" s="2">
@@ -8549,7 +8556,7 @@
         <v>83</v>
       </c>
       <c r="AF53" t="s" s="2">
-        <v>500</v>
+        <v>502</v>
       </c>
       <c r="AG53" t="s" s="2">
         <v>81</v>
@@ -8573,10 +8580,10 @@
         <v>83</v>
       </c>
       <c r="AN53" t="s" s="2">
-        <v>498</v>
+        <v>500</v>
       </c>
       <c r="AO53" t="s" s="2">
-        <v>505</v>
+        <v>507</v>
       </c>
       <c r="AP53" t="s" s="2">
         <v>83</v>
@@ -8587,10 +8594,10 @@
     </row>
     <row r="54">
       <c r="A54" t="s" s="2">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="B54" t="s" s="2">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="C54" s="2"/>
       <c r="D54" t="s" s="2">
@@ -8613,19 +8620,19 @@
         <v>96</v>
       </c>
       <c r="K54" t="s" s="2">
-        <v>441</v>
+        <v>443</v>
       </c>
       <c r="L54" t="s" s="2">
-        <v>507</v>
+        <v>509</v>
       </c>
       <c r="M54" t="s" s="2">
-        <v>508</v>
+        <v>510</v>
       </c>
       <c r="N54" t="s" s="2">
-        <v>509</v>
+        <v>511</v>
       </c>
       <c r="O54" t="s" s="2">
-        <v>510</v>
+        <v>512</v>
       </c>
       <c r="P54" t="s" s="2">
         <v>83</v>
@@ -8674,7 +8681,7 @@
         <v>83</v>
       </c>
       <c r="AF54" t="s" s="2">
-        <v>506</v>
+        <v>508</v>
       </c>
       <c r="AG54" t="s" s="2">
         <v>81</v>
@@ -8698,10 +8705,10 @@
         <v>83</v>
       </c>
       <c r="AN54" t="s" s="2">
-        <v>511</v>
+        <v>513</v>
       </c>
       <c r="AO54" t="s" s="2">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="AP54" t="s" s="2">
         <v>83</v>
@@ -8712,10 +8719,10 @@
     </row>
     <row r="55">
       <c r="A55" t="s" s="2">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="B55" t="s" s="2">
-        <v>513</v>
+        <v>515</v>
       </c>
       <c r="C55" s="2"/>
       <c r="D55" t="s" s="2">
@@ -8738,13 +8745,13 @@
         <v>83</v>
       </c>
       <c r="K55" t="s" s="2">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="L55" t="s" s="2">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="M55" t="s" s="2">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="N55" s="2"/>
       <c r="O55" s="2"/>
@@ -8795,7 +8802,7 @@
         <v>83</v>
       </c>
       <c r="AF55" t="s" s="2">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="AG55" t="s" s="2">
         <v>81</v>
@@ -8822,7 +8829,7 @@
         <v>83</v>
       </c>
       <c r="AO55" t="s" s="2">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="AP55" t="s" s="2">
         <v>83</v>
@@ -8833,10 +8840,10 @@
     </row>
     <row r="56">
       <c r="A56" t="s" s="2">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="B56" t="s" s="2">
-        <v>514</v>
+        <v>516</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" t="s" s="2">
@@ -8862,10 +8869,10 @@
         <v>140</v>
       </c>
       <c r="L56" t="s" s="2">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="M56" t="s" s="2">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="N56" t="s" s="2">
         <v>158</v>
@@ -8918,7 +8925,7 @@
         <v>83</v>
       </c>
       <c r="AF56" t="s" s="2">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="AG56" t="s" s="2">
         <v>81</v>
@@ -8945,7 +8952,7 @@
         <v>83</v>
       </c>
       <c r="AO56" t="s" s="2">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="AP56" t="s" s="2">
         <v>83</v>
@@ -8956,14 +8963,14 @@
     </row>
     <row r="57">
       <c r="A57" t="s" s="2">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="B57" t="s" s="2">
-        <v>515</v>
+        <v>517</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" t="s" s="2">
-        <v>452</v>
+        <v>454</v>
       </c>
       <c r="E57" s="2"/>
       <c r="F57" t="s" s="2">
@@ -8985,10 +8992,10 @@
         <v>140</v>
       </c>
       <c r="L57" t="s" s="2">
-        <v>453</v>
+        <v>455</v>
       </c>
       <c r="M57" t="s" s="2">
-        <v>454</v>
+        <v>456</v>
       </c>
       <c r="N57" t="s" s="2">
         <v>158</v>
@@ -9043,7 +9050,7 @@
         <v>83</v>
       </c>
       <c r="AF57" t="s" s="2">
-        <v>455</v>
+        <v>457</v>
       </c>
       <c r="AG57" t="s" s="2">
         <v>81</v>
@@ -9081,10 +9088,10 @@
     </row>
     <row r="58">
       <c r="A58" t="s" s="2">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="B58" t="s" s="2">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" t="s" s="2">
@@ -9107,19 +9114,19 @@
         <v>96</v>
       </c>
       <c r="K58" t="s" s="2">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="L58" t="s" s="2">
-        <v>517</v>
+        <v>519</v>
       </c>
       <c r="M58" t="s" s="2">
-        <v>518</v>
+        <v>520</v>
       </c>
       <c r="N58" t="s" s="2">
-        <v>519</v>
+        <v>521</v>
       </c>
       <c r="O58" t="s" s="2">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="P58" t="s" s="2">
         <v>83</v>
@@ -9144,13 +9151,13 @@
         <v>83</v>
       </c>
       <c r="X58" t="s" s="2">
-        <v>293</v>
+        <v>295</v>
       </c>
       <c r="Y58" t="s" s="2">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="Z58" t="s" s="2">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="AA58" t="s" s="2">
         <v>83</v>
@@ -9168,7 +9175,7 @@
         <v>83</v>
       </c>
       <c r="AF58" t="s" s="2">
-        <v>516</v>
+        <v>518</v>
       </c>
       <c r="AG58" t="s" s="2">
         <v>95</v>
@@ -9189,16 +9196,16 @@
         <v>83</v>
       </c>
       <c r="AM58" t="s" s="2">
-        <v>520</v>
+        <v>522</v>
       </c>
       <c r="AN58" t="s" s="2">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="AO58" t="s" s="2">
-        <v>299</v>
+        <v>301</v>
       </c>
       <c r="AP58" t="s" s="2">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="AQ58" t="s" s="2">
         <v>83</v>
@@ -9206,10 +9213,10 @@
     </row>
     <row r="59">
       <c r="A59" t="s" s="2">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="B59" t="s" s="2">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="C59" s="2"/>
       <c r="D59" t="s" s="2">
@@ -9232,19 +9239,19 @@
         <v>96</v>
       </c>
       <c r="K59" t="s" s="2">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="L59" t="s" s="2">
-        <v>522</v>
+        <v>524</v>
       </c>
       <c r="M59" t="s" s="2">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="N59" t="s" s="2">
-        <v>523</v>
+        <v>525</v>
       </c>
       <c r="O59" t="s" s="2">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="P59" t="s" s="2">
         <v>83</v>
@@ -9293,7 +9300,7 @@
         <v>83</v>
       </c>
       <c r="AF59" t="s" s="2">
-        <v>521</v>
+        <v>523</v>
       </c>
       <c r="AG59" t="s" s="2">
         <v>81</v>
@@ -9314,27 +9321,27 @@
         <v>83</v>
       </c>
       <c r="AM59" t="s" s="2">
-        <v>524</v>
+        <v>526</v>
       </c>
       <c r="AN59" t="s" s="2">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="AO59" t="s" s="2">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="AP59" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AQ59" t="s" s="2">
-        <v>373</v>
+        <v>375</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="s" s="2">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="B60" t="s" s="2">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="C60" s="2"/>
       <c r="D60" t="s" s="2">
@@ -9357,19 +9364,19 @@
         <v>83</v>
       </c>
       <c r="K60" t="s" s="2">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="L60" t="s" s="2">
-        <v>526</v>
+        <v>528</v>
       </c>
       <c r="M60" t="s" s="2">
-        <v>527</v>
+        <v>529</v>
       </c>
       <c r="N60" t="s" s="2">
-        <v>528</v>
+        <v>530</v>
       </c>
       <c r="O60" t="s" s="2">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="P60" t="s" s="2">
         <v>83</v>
@@ -9394,13 +9401,13 @@
         <v>83</v>
       </c>
       <c r="X60" t="s" s="2">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="Y60" t="s" s="2">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="Z60" t="s" s="2">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="AA60" t="s" s="2">
         <v>83</v>
@@ -9418,7 +9425,7 @@
         <v>83</v>
       </c>
       <c r="AF60" t="s" s="2">
-        <v>525</v>
+        <v>527</v>
       </c>
       <c r="AG60" t="s" s="2">
         <v>81</v>
@@ -9427,7 +9434,7 @@
         <v>95</v>
       </c>
       <c r="AI60" t="s" s="2">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="AJ60" t="s" s="2">
         <v>107</v>
@@ -9445,7 +9452,7 @@
         <v>138</v>
       </c>
       <c r="AO60" t="s" s="2">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="AP60" t="s" s="2">
         <v>83</v>
@@ -9456,14 +9463,14 @@
     </row>
     <row r="61">
       <c r="A61" t="s" s="2">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="B61" t="s" s="2">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" t="s" s="2">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="E61" s="2"/>
       <c r="F61" t="s" s="2">
@@ -9482,19 +9489,19 @@
         <v>83</v>
       </c>
       <c r="K61" t="s" s="2">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="L61" t="s" s="2">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="M61" t="s" s="2">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="N61" t="s" s="2">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="O61" t="s" s="2">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="P61" t="s" s="2">
         <v>83</v>
@@ -9519,13 +9526,13 @@
         <v>83</v>
       </c>
       <c r="X61" t="s" s="2">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="Y61" t="s" s="2">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="Z61" t="s" s="2">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="AA61" t="s" s="2">
         <v>83</v>
@@ -9543,7 +9550,7 @@
         <v>83</v>
       </c>
       <c r="AF61" t="s" s="2">
-        <v>529</v>
+        <v>531</v>
       </c>
       <c r="AG61" t="s" s="2">
         <v>81</v>
@@ -9564,27 +9571,27 @@
         <v>83</v>
       </c>
       <c r="AM61" t="s" s="2">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="AN61" t="s" s="2">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="AO61" t="s" s="2">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="AP61" t="s" s="2">
         <v>83</v>
       </c>
       <c r="AQ61" t="s" s="2">
-        <v>394</v>
+        <v>396</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="s" s="2">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="B62" t="s" s="2">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="C62" s="2"/>
       <c r="D62" t="s" s="2">
@@ -9610,16 +9617,16 @@
         <v>84</v>
       </c>
       <c r="L62" t="s" s="2">
-        <v>531</v>
+        <v>533</v>
       </c>
       <c r="M62" t="s" s="2">
-        <v>532</v>
+        <v>534</v>
       </c>
       <c r="N62" t="s" s="2">
-        <v>444</v>
+        <v>446</v>
       </c>
       <c r="O62" t="s" s="2">
-        <v>445</v>
+        <v>447</v>
       </c>
       <c r="P62" t="s" s="2">
         <v>83</v>
@@ -9668,7 +9675,7 @@
         <v>83</v>
       </c>
       <c r="AF62" t="s" s="2">
-        <v>530</v>
+        <v>532</v>
       </c>
       <c r="AG62" t="s" s="2">
         <v>81</v>
@@ -9692,10 +9699,10 @@
         <v>83</v>
       </c>
       <c r="AN62" t="s" s="2">
-        <v>447</v>
+        <v>449</v>
       </c>
       <c r="AO62" t="s" s="2">
-        <v>448</v>
+        <v>450</v>
       </c>
       <c r="AP62" t="s" s="2">
         <v>83</v>

</xml_diff>